<commit_message>
feat: support question images in exams
</commit_message>
<xml_diff>
--- a/front-end/assets/templates/modelo-importacao-questoes.xlsx
+++ b/front-end/assets/templates/modelo-importacao-questoes.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questões" sheetId="1" r:id="R35b1b138c9e04a01"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instruções" sheetId="2" r:id="Re5bd3fbcc8994e18"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exemplos" sheetId="3" r:id="Rd646cc7babec4504"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questões" sheetId="1" r:id="R2188f67087d442aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instruções" sheetId="2" r:id="Ra283d2d89f5540bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exemplos" sheetId="3" r:id="R56303d2fa9d9498a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -59,7 +59,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="9">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -89,6 +89,11 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFF8FAFC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF4FBFF"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -318,7 +323,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="100">
+  <x:cellXfs count="103">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -450,13 +455,22 @@
     <x:xf numFmtId="0" fontId="4" fillId="6" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="4" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -549,12 +563,12 @@
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="6" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -773,7 +787,9 @@
     <x:col min="12" max="12" width="24" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="24" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="24" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="26" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="42" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="32" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="26" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -794,6 +810,8 @@
       <x:c r="M1" s="4"/>
       <x:c r="N1" s="4"/>
       <x:c r="O1" s="4"/>
+      <x:c r="P1" s="4"/>
+      <x:c r="Q1" s="4"/>
     </x:row>
     <x:row r="2" ht="27" customHeight="1">
       <x:c r="A2" s="8" t="str">
@@ -813,6 +831,8 @@
       <x:c r="M2" s="8"/>
       <x:c r="N2" s="8"/>
       <x:c r="O2" s="8"/>
+      <x:c r="P2" s="8"/>
+      <x:c r="Q2" s="8"/>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="20" t="str">
@@ -857,14 +877,20 @@
       <x:c r="N4" s="21" t="str">
         <x:v>Alternativa J</x:v>
       </x:c>
-      <x:c r="O4" s="22" t="str">
+      <x:c r="O4" s="21" t="str">
+        <x:v>Imagem</x:v>
+      </x:c>
+      <x:c r="P4" s="21" t="str">
+        <x:v>Texto alternativo</x:v>
+      </x:c>
+      <x:c r="Q4" s="22" t="str">
         <x:v>Resposta correta</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="51"/>
       <x:c r="B5" s="43"/>
-      <x:c r="C5" s="60"/>
+      <x:c r="C5" s="63"/>
       <x:c r="D5" s="54"/>
       <x:c r="E5" s="43"/>
       <x:c r="F5" s="43"/>
@@ -877,11 +903,13 @@
       <x:c r="M5" s="43"/>
       <x:c r="N5" s="43"/>
       <x:c r="O5" s="57"/>
+      <x:c r="P5" s="57"/>
+      <x:c r="Q5" s="60"/>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="52"/>
       <x:c r="B6" s="46"/>
-      <x:c r="C6" s="61"/>
+      <x:c r="C6" s="64"/>
       <x:c r="D6" s="55"/>
       <x:c r="E6" s="46"/>
       <x:c r="F6" s="46"/>
@@ -894,11 +922,13 @@
       <x:c r="M6" s="46"/>
       <x:c r="N6" s="46"/>
       <x:c r="O6" s="58"/>
+      <x:c r="P6" s="58"/>
+      <x:c r="Q6" s="61"/>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="52"/>
       <x:c r="B7" s="46"/>
-      <x:c r="C7" s="61"/>
+      <x:c r="C7" s="64"/>
       <x:c r="D7" s="55"/>
       <x:c r="E7" s="46"/>
       <x:c r="F7" s="46"/>
@@ -911,11 +941,13 @@
       <x:c r="M7" s="46"/>
       <x:c r="N7" s="46"/>
       <x:c r="O7" s="58"/>
+      <x:c r="P7" s="58"/>
+      <x:c r="Q7" s="61"/>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="52"/>
       <x:c r="B8" s="46"/>
-      <x:c r="C8" s="61"/>
+      <x:c r="C8" s="64"/>
       <x:c r="D8" s="55"/>
       <x:c r="E8" s="46"/>
       <x:c r="F8" s="46"/>
@@ -928,11 +960,13 @@
       <x:c r="M8" s="46"/>
       <x:c r="N8" s="46"/>
       <x:c r="O8" s="58"/>
+      <x:c r="P8" s="58"/>
+      <x:c r="Q8" s="61"/>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="52"/>
       <x:c r="B9" s="46"/>
-      <x:c r="C9" s="61"/>
+      <x:c r="C9" s="64"/>
       <x:c r="D9" s="55"/>
       <x:c r="E9" s="46"/>
       <x:c r="F9" s="46"/>
@@ -945,11 +979,13 @@
       <x:c r="M9" s="46"/>
       <x:c r="N9" s="46"/>
       <x:c r="O9" s="58"/>
+      <x:c r="P9" s="58"/>
+      <x:c r="Q9" s="61"/>
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="52"/>
       <x:c r="B10" s="46"/>
-      <x:c r="C10" s="61"/>
+      <x:c r="C10" s="64"/>
       <x:c r="D10" s="55"/>
       <x:c r="E10" s="46"/>
       <x:c r="F10" s="46"/>
@@ -962,11 +998,13 @@
       <x:c r="M10" s="46"/>
       <x:c r="N10" s="46"/>
       <x:c r="O10" s="58"/>
+      <x:c r="P10" s="58"/>
+      <x:c r="Q10" s="61"/>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="52"/>
       <x:c r="B11" s="46"/>
-      <x:c r="C11" s="61"/>
+      <x:c r="C11" s="64"/>
       <x:c r="D11" s="55"/>
       <x:c r="E11" s="46"/>
       <x:c r="F11" s="46"/>
@@ -979,11 +1017,13 @@
       <x:c r="M11" s="46"/>
       <x:c r="N11" s="46"/>
       <x:c r="O11" s="58"/>
+      <x:c r="P11" s="58"/>
+      <x:c r="Q11" s="61"/>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="52"/>
       <x:c r="B12" s="46"/>
-      <x:c r="C12" s="61"/>
+      <x:c r="C12" s="64"/>
       <x:c r="D12" s="55"/>
       <x:c r="E12" s="46"/>
       <x:c r="F12" s="46"/>
@@ -996,11 +1036,13 @@
       <x:c r="M12" s="46"/>
       <x:c r="N12" s="46"/>
       <x:c r="O12" s="58"/>
+      <x:c r="P12" s="58"/>
+      <x:c r="Q12" s="61"/>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="52"/>
       <x:c r="B13" s="46"/>
-      <x:c r="C13" s="61"/>
+      <x:c r="C13" s="64"/>
       <x:c r="D13" s="55"/>
       <x:c r="E13" s="46"/>
       <x:c r="F13" s="46"/>
@@ -1013,11 +1055,13 @@
       <x:c r="M13" s="46"/>
       <x:c r="N13" s="46"/>
       <x:c r="O13" s="58"/>
+      <x:c r="P13" s="58"/>
+      <x:c r="Q13" s="61"/>
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="52"/>
       <x:c r="B14" s="46"/>
-      <x:c r="C14" s="61"/>
+      <x:c r="C14" s="64"/>
       <x:c r="D14" s="55"/>
       <x:c r="E14" s="46"/>
       <x:c r="F14" s="46"/>
@@ -1030,11 +1074,13 @@
       <x:c r="M14" s="46"/>
       <x:c r="N14" s="46"/>
       <x:c r="O14" s="58"/>
+      <x:c r="P14" s="58"/>
+      <x:c r="Q14" s="61"/>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="52"/>
       <x:c r="B15" s="46"/>
-      <x:c r="C15" s="61"/>
+      <x:c r="C15" s="64"/>
       <x:c r="D15" s="55"/>
       <x:c r="E15" s="46"/>
       <x:c r="F15" s="46"/>
@@ -1047,11 +1093,13 @@
       <x:c r="M15" s="46"/>
       <x:c r="N15" s="46"/>
       <x:c r="O15" s="58"/>
+      <x:c r="P15" s="58"/>
+      <x:c r="Q15" s="61"/>
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="52"/>
       <x:c r="B16" s="46"/>
-      <x:c r="C16" s="61"/>
+      <x:c r="C16" s="64"/>
       <x:c r="D16" s="55"/>
       <x:c r="E16" s="46"/>
       <x:c r="F16" s="46"/>
@@ -1064,11 +1112,13 @@
       <x:c r="M16" s="46"/>
       <x:c r="N16" s="46"/>
       <x:c r="O16" s="58"/>
+      <x:c r="P16" s="58"/>
+      <x:c r="Q16" s="61"/>
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="52"/>
       <x:c r="B17" s="46"/>
-      <x:c r="C17" s="61"/>
+      <x:c r="C17" s="64"/>
       <x:c r="D17" s="55"/>
       <x:c r="E17" s="46"/>
       <x:c r="F17" s="46"/>
@@ -1081,11 +1131,13 @@
       <x:c r="M17" s="46"/>
       <x:c r="N17" s="46"/>
       <x:c r="O17" s="58"/>
+      <x:c r="P17" s="58"/>
+      <x:c r="Q17" s="61"/>
     </x:row>
     <x:row r="18" ht="15" hidden="0" customHeight="1">
       <x:c r="A18" s="52"/>
       <x:c r="B18" s="46"/>
-      <x:c r="C18" s="61"/>
+      <x:c r="C18" s="64"/>
       <x:c r="D18" s="55"/>
       <x:c r="E18" s="46"/>
       <x:c r="F18" s="46"/>
@@ -1098,11 +1150,13 @@
       <x:c r="M18" s="46"/>
       <x:c r="N18" s="46"/>
       <x:c r="O18" s="58"/>
+      <x:c r="P18" s="58"/>
+      <x:c r="Q18" s="61"/>
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
       <x:c r="A19" s="52"/>
       <x:c r="B19" s="46"/>
-      <x:c r="C19" s="61"/>
+      <x:c r="C19" s="64"/>
       <x:c r="D19" s="55"/>
       <x:c r="E19" s="46"/>
       <x:c r="F19" s="46"/>
@@ -1115,11 +1169,13 @@
       <x:c r="M19" s="46"/>
       <x:c r="N19" s="46"/>
       <x:c r="O19" s="58"/>
+      <x:c r="P19" s="58"/>
+      <x:c r="Q19" s="61"/>
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
       <x:c r="A20" s="52"/>
       <x:c r="B20" s="46"/>
-      <x:c r="C20" s="61"/>
+      <x:c r="C20" s="64"/>
       <x:c r="D20" s="55"/>
       <x:c r="E20" s="46"/>
       <x:c r="F20" s="46"/>
@@ -1132,11 +1188,13 @@
       <x:c r="M20" s="46"/>
       <x:c r="N20" s="46"/>
       <x:c r="O20" s="58"/>
+      <x:c r="P20" s="58"/>
+      <x:c r="Q20" s="61"/>
     </x:row>
     <x:row r="21" ht="15" hidden="0" customHeight="1">
       <x:c r="A21" s="52"/>
       <x:c r="B21" s="46"/>
-      <x:c r="C21" s="61"/>
+      <x:c r="C21" s="64"/>
       <x:c r="D21" s="55"/>
       <x:c r="E21" s="46"/>
       <x:c r="F21" s="46"/>
@@ -1149,11 +1207,13 @@
       <x:c r="M21" s="46"/>
       <x:c r="N21" s="46"/>
       <x:c r="O21" s="58"/>
+      <x:c r="P21" s="58"/>
+      <x:c r="Q21" s="61"/>
     </x:row>
     <x:row r="22" ht="15" hidden="0" customHeight="1">
       <x:c r="A22" s="52"/>
       <x:c r="B22" s="46"/>
-      <x:c r="C22" s="61"/>
+      <x:c r="C22" s="64"/>
       <x:c r="D22" s="55"/>
       <x:c r="E22" s="46"/>
       <x:c r="F22" s="46"/>
@@ -1166,11 +1226,13 @@
       <x:c r="M22" s="46"/>
       <x:c r="N22" s="46"/>
       <x:c r="O22" s="58"/>
+      <x:c r="P22" s="58"/>
+      <x:c r="Q22" s="61"/>
     </x:row>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
       <x:c r="A23" s="52"/>
       <x:c r="B23" s="46"/>
-      <x:c r="C23" s="61"/>
+      <x:c r="C23" s="64"/>
       <x:c r="D23" s="55"/>
       <x:c r="E23" s="46"/>
       <x:c r="F23" s="46"/>
@@ -1183,11 +1245,13 @@
       <x:c r="M23" s="46"/>
       <x:c r="N23" s="46"/>
       <x:c r="O23" s="58"/>
+      <x:c r="P23" s="58"/>
+      <x:c r="Q23" s="61"/>
     </x:row>
     <x:row r="24" ht="15" hidden="0" customHeight="1">
       <x:c r="A24" s="52"/>
       <x:c r="B24" s="46"/>
-      <x:c r="C24" s="61"/>
+      <x:c r="C24" s="64"/>
       <x:c r="D24" s="55"/>
       <x:c r="E24" s="46"/>
       <x:c r="F24" s="46"/>
@@ -1200,11 +1264,13 @@
       <x:c r="M24" s="46"/>
       <x:c r="N24" s="46"/>
       <x:c r="O24" s="58"/>
+      <x:c r="P24" s="58"/>
+      <x:c r="Q24" s="61"/>
     </x:row>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
       <x:c r="A25" s="52"/>
       <x:c r="B25" s="46"/>
-      <x:c r="C25" s="61"/>
+      <x:c r="C25" s="64"/>
       <x:c r="D25" s="55"/>
       <x:c r="E25" s="46"/>
       <x:c r="F25" s="46"/>
@@ -1217,11 +1283,13 @@
       <x:c r="M25" s="46"/>
       <x:c r="N25" s="46"/>
       <x:c r="O25" s="58"/>
+      <x:c r="P25" s="58"/>
+      <x:c r="Q25" s="61"/>
     </x:row>
     <x:row r="26" ht="15" hidden="0" customHeight="1">
       <x:c r="A26" s="52"/>
       <x:c r="B26" s="46"/>
-      <x:c r="C26" s="61"/>
+      <x:c r="C26" s="64"/>
       <x:c r="D26" s="55"/>
       <x:c r="E26" s="46"/>
       <x:c r="F26" s="46"/>
@@ -1234,11 +1302,13 @@
       <x:c r="M26" s="46"/>
       <x:c r="N26" s="46"/>
       <x:c r="O26" s="58"/>
+      <x:c r="P26" s="58"/>
+      <x:c r="Q26" s="61"/>
     </x:row>
     <x:row r="27" ht="15" hidden="0" customHeight="1">
       <x:c r="A27" s="52"/>
       <x:c r="B27" s="46"/>
-      <x:c r="C27" s="61"/>
+      <x:c r="C27" s="64"/>
       <x:c r="D27" s="55"/>
       <x:c r="E27" s="46"/>
       <x:c r="F27" s="46"/>
@@ -1251,11 +1321,13 @@
       <x:c r="M27" s="46"/>
       <x:c r="N27" s="46"/>
       <x:c r="O27" s="58"/>
+      <x:c r="P27" s="58"/>
+      <x:c r="Q27" s="61"/>
     </x:row>
     <x:row r="28" ht="15" hidden="0" customHeight="1">
       <x:c r="A28" s="52"/>
       <x:c r="B28" s="46"/>
-      <x:c r="C28" s="61"/>
+      <x:c r="C28" s="64"/>
       <x:c r="D28" s="55"/>
       <x:c r="E28" s="46"/>
       <x:c r="F28" s="46"/>
@@ -1268,11 +1340,13 @@
       <x:c r="M28" s="46"/>
       <x:c r="N28" s="46"/>
       <x:c r="O28" s="58"/>
+      <x:c r="P28" s="58"/>
+      <x:c r="Q28" s="61"/>
     </x:row>
     <x:row r="29" ht="15" hidden="0" customHeight="1">
       <x:c r="A29" s="52"/>
       <x:c r="B29" s="46"/>
-      <x:c r="C29" s="61"/>
+      <x:c r="C29" s="64"/>
       <x:c r="D29" s="55"/>
       <x:c r="E29" s="46"/>
       <x:c r="F29" s="46"/>
@@ -1285,11 +1359,13 @@
       <x:c r="M29" s="46"/>
       <x:c r="N29" s="46"/>
       <x:c r="O29" s="58"/>
+      <x:c r="P29" s="58"/>
+      <x:c r="Q29" s="61"/>
     </x:row>
     <x:row r="30" ht="15" hidden="0" customHeight="1">
       <x:c r="A30" s="52"/>
       <x:c r="B30" s="46"/>
-      <x:c r="C30" s="61"/>
+      <x:c r="C30" s="64"/>
       <x:c r="D30" s="55"/>
       <x:c r="E30" s="46"/>
       <x:c r="F30" s="46"/>
@@ -1302,11 +1378,13 @@
       <x:c r="M30" s="46"/>
       <x:c r="N30" s="46"/>
       <x:c r="O30" s="58"/>
+      <x:c r="P30" s="58"/>
+      <x:c r="Q30" s="61"/>
     </x:row>
     <x:row r="31" ht="15" hidden="0" customHeight="1">
       <x:c r="A31" s="52"/>
       <x:c r="B31" s="46"/>
-      <x:c r="C31" s="61"/>
+      <x:c r="C31" s="64"/>
       <x:c r="D31" s="55"/>
       <x:c r="E31" s="46"/>
       <x:c r="F31" s="46"/>
@@ -1319,11 +1397,13 @@
       <x:c r="M31" s="46"/>
       <x:c r="N31" s="46"/>
       <x:c r="O31" s="58"/>
+      <x:c r="P31" s="58"/>
+      <x:c r="Q31" s="61"/>
     </x:row>
     <x:row r="32" ht="15" hidden="0" customHeight="1">
       <x:c r="A32" s="52"/>
       <x:c r="B32" s="46"/>
-      <x:c r="C32" s="61"/>
+      <x:c r="C32" s="64"/>
       <x:c r="D32" s="55"/>
       <x:c r="E32" s="46"/>
       <x:c r="F32" s="46"/>
@@ -1336,11 +1416,13 @@
       <x:c r="M32" s="46"/>
       <x:c r="N32" s="46"/>
       <x:c r="O32" s="58"/>
+      <x:c r="P32" s="58"/>
+      <x:c r="Q32" s="61"/>
     </x:row>
     <x:row r="33" ht="15" hidden="0" customHeight="1">
       <x:c r="A33" s="52"/>
       <x:c r="B33" s="46"/>
-      <x:c r="C33" s="61"/>
+      <x:c r="C33" s="64"/>
       <x:c r="D33" s="55"/>
       <x:c r="E33" s="46"/>
       <x:c r="F33" s="46"/>
@@ -1353,11 +1435,13 @@
       <x:c r="M33" s="46"/>
       <x:c r="N33" s="46"/>
       <x:c r="O33" s="58"/>
+      <x:c r="P33" s="58"/>
+      <x:c r="Q33" s="61"/>
     </x:row>
     <x:row r="34" ht="15" hidden="0" customHeight="1">
       <x:c r="A34" s="52"/>
       <x:c r="B34" s="46"/>
-      <x:c r="C34" s="61"/>
+      <x:c r="C34" s="64"/>
       <x:c r="D34" s="55"/>
       <x:c r="E34" s="46"/>
       <x:c r="F34" s="46"/>
@@ -1370,11 +1454,13 @@
       <x:c r="M34" s="46"/>
       <x:c r="N34" s="46"/>
       <x:c r="O34" s="58"/>
+      <x:c r="P34" s="58"/>
+      <x:c r="Q34" s="61"/>
     </x:row>
     <x:row r="35" ht="15" hidden="0" customHeight="1">
       <x:c r="A35" s="52"/>
       <x:c r="B35" s="46"/>
-      <x:c r="C35" s="61"/>
+      <x:c r="C35" s="64"/>
       <x:c r="D35" s="55"/>
       <x:c r="E35" s="46"/>
       <x:c r="F35" s="46"/>
@@ -1387,11 +1473,13 @@
       <x:c r="M35" s="46"/>
       <x:c r="N35" s="46"/>
       <x:c r="O35" s="58"/>
+      <x:c r="P35" s="58"/>
+      <x:c r="Q35" s="61"/>
     </x:row>
     <x:row r="36" ht="15" hidden="0" customHeight="1">
       <x:c r="A36" s="52"/>
       <x:c r="B36" s="46"/>
-      <x:c r="C36" s="61"/>
+      <x:c r="C36" s="64"/>
       <x:c r="D36" s="55"/>
       <x:c r="E36" s="46"/>
       <x:c r="F36" s="46"/>
@@ -1404,11 +1492,13 @@
       <x:c r="M36" s="46"/>
       <x:c r="N36" s="46"/>
       <x:c r="O36" s="58"/>
+      <x:c r="P36" s="58"/>
+      <x:c r="Q36" s="61"/>
     </x:row>
     <x:row r="37" ht="15" hidden="0" customHeight="1">
       <x:c r="A37" s="52"/>
       <x:c r="B37" s="46"/>
-      <x:c r="C37" s="61"/>
+      <x:c r="C37" s="64"/>
       <x:c r="D37" s="55"/>
       <x:c r="E37" s="46"/>
       <x:c r="F37" s="46"/>
@@ -1421,11 +1511,13 @@
       <x:c r="M37" s="46"/>
       <x:c r="N37" s="46"/>
       <x:c r="O37" s="58"/>
+      <x:c r="P37" s="58"/>
+      <x:c r="Q37" s="61"/>
     </x:row>
     <x:row r="38" ht="15" hidden="0" customHeight="1">
       <x:c r="A38" s="52"/>
       <x:c r="B38" s="46"/>
-      <x:c r="C38" s="61"/>
+      <x:c r="C38" s="64"/>
       <x:c r="D38" s="55"/>
       <x:c r="E38" s="46"/>
       <x:c r="F38" s="46"/>
@@ -1438,11 +1530,13 @@
       <x:c r="M38" s="46"/>
       <x:c r="N38" s="46"/>
       <x:c r="O38" s="58"/>
+      <x:c r="P38" s="58"/>
+      <x:c r="Q38" s="61"/>
     </x:row>
     <x:row r="39" ht="15" hidden="0" customHeight="1">
       <x:c r="A39" s="52"/>
       <x:c r="B39" s="46"/>
-      <x:c r="C39" s="61"/>
+      <x:c r="C39" s="64"/>
       <x:c r="D39" s="55"/>
       <x:c r="E39" s="46"/>
       <x:c r="F39" s="46"/>
@@ -1455,11 +1549,13 @@
       <x:c r="M39" s="46"/>
       <x:c r="N39" s="46"/>
       <x:c r="O39" s="58"/>
+      <x:c r="P39" s="58"/>
+      <x:c r="Q39" s="61"/>
     </x:row>
     <x:row r="40" ht="15" hidden="0" customHeight="1">
       <x:c r="A40" s="52"/>
       <x:c r="B40" s="46"/>
-      <x:c r="C40" s="61"/>
+      <x:c r="C40" s="64"/>
       <x:c r="D40" s="55"/>
       <x:c r="E40" s="46"/>
       <x:c r="F40" s="46"/>
@@ -1472,11 +1568,13 @@
       <x:c r="M40" s="46"/>
       <x:c r="N40" s="46"/>
       <x:c r="O40" s="58"/>
+      <x:c r="P40" s="58"/>
+      <x:c r="Q40" s="61"/>
     </x:row>
     <x:row r="41" ht="15" hidden="0" customHeight="1">
       <x:c r="A41" s="52"/>
       <x:c r="B41" s="46"/>
-      <x:c r="C41" s="61"/>
+      <x:c r="C41" s="64"/>
       <x:c r="D41" s="55"/>
       <x:c r="E41" s="46"/>
       <x:c r="F41" s="46"/>
@@ -1489,11 +1587,13 @@
       <x:c r="M41" s="46"/>
       <x:c r="N41" s="46"/>
       <x:c r="O41" s="58"/>
+      <x:c r="P41" s="58"/>
+      <x:c r="Q41" s="61"/>
     </x:row>
     <x:row r="42" ht="15" hidden="0" customHeight="1">
       <x:c r="A42" s="52"/>
       <x:c r="B42" s="46"/>
-      <x:c r="C42" s="61"/>
+      <x:c r="C42" s="64"/>
       <x:c r="D42" s="55"/>
       <x:c r="E42" s="46"/>
       <x:c r="F42" s="46"/>
@@ -1506,11 +1606,13 @@
       <x:c r="M42" s="46"/>
       <x:c r="N42" s="46"/>
       <x:c r="O42" s="58"/>
+      <x:c r="P42" s="58"/>
+      <x:c r="Q42" s="61"/>
     </x:row>
     <x:row r="43" ht="15" hidden="0" customHeight="1">
       <x:c r="A43" s="52"/>
       <x:c r="B43" s="46"/>
-      <x:c r="C43" s="61"/>
+      <x:c r="C43" s="64"/>
       <x:c r="D43" s="55"/>
       <x:c r="E43" s="46"/>
       <x:c r="F43" s="46"/>
@@ -1523,11 +1625,13 @@
       <x:c r="M43" s="46"/>
       <x:c r="N43" s="46"/>
       <x:c r="O43" s="58"/>
+      <x:c r="P43" s="58"/>
+      <x:c r="Q43" s="61"/>
     </x:row>
     <x:row r="44" ht="15" hidden="0" customHeight="1">
       <x:c r="A44" s="52"/>
       <x:c r="B44" s="46"/>
-      <x:c r="C44" s="61"/>
+      <x:c r="C44" s="64"/>
       <x:c r="D44" s="55"/>
       <x:c r="E44" s="46"/>
       <x:c r="F44" s="46"/>
@@ -1540,11 +1644,13 @@
       <x:c r="M44" s="46"/>
       <x:c r="N44" s="46"/>
       <x:c r="O44" s="58"/>
+      <x:c r="P44" s="58"/>
+      <x:c r="Q44" s="61"/>
     </x:row>
     <x:row r="45" ht="15" hidden="0" customHeight="1">
       <x:c r="A45" s="52"/>
       <x:c r="B45" s="46"/>
-      <x:c r="C45" s="61"/>
+      <x:c r="C45" s="64"/>
       <x:c r="D45" s="55"/>
       <x:c r="E45" s="46"/>
       <x:c r="F45" s="46"/>
@@ -1557,11 +1663,13 @@
       <x:c r="M45" s="46"/>
       <x:c r="N45" s="46"/>
       <x:c r="O45" s="58"/>
+      <x:c r="P45" s="58"/>
+      <x:c r="Q45" s="61"/>
     </x:row>
     <x:row r="46" ht="15" hidden="0" customHeight="1">
       <x:c r="A46" s="52"/>
       <x:c r="B46" s="46"/>
-      <x:c r="C46" s="61"/>
+      <x:c r="C46" s="64"/>
       <x:c r="D46" s="55"/>
       <x:c r="E46" s="46"/>
       <x:c r="F46" s="46"/>
@@ -1574,11 +1682,13 @@
       <x:c r="M46" s="46"/>
       <x:c r="N46" s="46"/>
       <x:c r="O46" s="58"/>
+      <x:c r="P46" s="58"/>
+      <x:c r="Q46" s="61"/>
     </x:row>
     <x:row r="47" ht="15" hidden="0" customHeight="1">
       <x:c r="A47" s="52"/>
       <x:c r="B47" s="46"/>
-      <x:c r="C47" s="61"/>
+      <x:c r="C47" s="64"/>
       <x:c r="D47" s="55"/>
       <x:c r="E47" s="46"/>
       <x:c r="F47" s="46"/>
@@ -1591,11 +1701,13 @@
       <x:c r="M47" s="46"/>
       <x:c r="N47" s="46"/>
       <x:c r="O47" s="58"/>
+      <x:c r="P47" s="58"/>
+      <x:c r="Q47" s="61"/>
     </x:row>
     <x:row r="48" ht="15" hidden="0" customHeight="1">
       <x:c r="A48" s="52"/>
       <x:c r="B48" s="46"/>
-      <x:c r="C48" s="61"/>
+      <x:c r="C48" s="64"/>
       <x:c r="D48" s="55"/>
       <x:c r="E48" s="46"/>
       <x:c r="F48" s="46"/>
@@ -1608,11 +1720,13 @@
       <x:c r="M48" s="46"/>
       <x:c r="N48" s="46"/>
       <x:c r="O48" s="58"/>
+      <x:c r="P48" s="58"/>
+      <x:c r="Q48" s="61"/>
     </x:row>
     <x:row r="49" ht="15" hidden="0" customHeight="1">
       <x:c r="A49" s="52"/>
       <x:c r="B49" s="46"/>
-      <x:c r="C49" s="61"/>
+      <x:c r="C49" s="64"/>
       <x:c r="D49" s="55"/>
       <x:c r="E49" s="46"/>
       <x:c r="F49" s="46"/>
@@ -1625,11 +1739,13 @@
       <x:c r="M49" s="46"/>
       <x:c r="N49" s="46"/>
       <x:c r="O49" s="58"/>
+      <x:c r="P49" s="58"/>
+      <x:c r="Q49" s="61"/>
     </x:row>
     <x:row r="50" ht="15" hidden="0" customHeight="1">
       <x:c r="A50" s="52"/>
       <x:c r="B50" s="46"/>
-      <x:c r="C50" s="61"/>
+      <x:c r="C50" s="64"/>
       <x:c r="D50" s="55"/>
       <x:c r="E50" s="46"/>
       <x:c r="F50" s="46"/>
@@ -1642,11 +1758,13 @@
       <x:c r="M50" s="46"/>
       <x:c r="N50" s="46"/>
       <x:c r="O50" s="58"/>
+      <x:c r="P50" s="58"/>
+      <x:c r="Q50" s="61"/>
     </x:row>
     <x:row r="51" ht="15" hidden="0" customHeight="1">
       <x:c r="A51" s="52"/>
       <x:c r="B51" s="46"/>
-      <x:c r="C51" s="61"/>
+      <x:c r="C51" s="64"/>
       <x:c r="D51" s="55"/>
       <x:c r="E51" s="46"/>
       <x:c r="F51" s="46"/>
@@ -1659,11 +1777,13 @@
       <x:c r="M51" s="46"/>
       <x:c r="N51" s="46"/>
       <x:c r="O51" s="58"/>
+      <x:c r="P51" s="58"/>
+      <x:c r="Q51" s="61"/>
     </x:row>
     <x:row r="52" ht="15" hidden="0" customHeight="1">
       <x:c r="A52" s="52"/>
       <x:c r="B52" s="46"/>
-      <x:c r="C52" s="61"/>
+      <x:c r="C52" s="64"/>
       <x:c r="D52" s="55"/>
       <x:c r="E52" s="46"/>
       <x:c r="F52" s="46"/>
@@ -1676,11 +1796,13 @@
       <x:c r="M52" s="46"/>
       <x:c r="N52" s="46"/>
       <x:c r="O52" s="58"/>
+      <x:c r="P52" s="58"/>
+      <x:c r="Q52" s="61"/>
     </x:row>
     <x:row r="53" ht="15" hidden="0" customHeight="1">
       <x:c r="A53" s="52"/>
       <x:c r="B53" s="46"/>
-      <x:c r="C53" s="61"/>
+      <x:c r="C53" s="64"/>
       <x:c r="D53" s="55"/>
       <x:c r="E53" s="46"/>
       <x:c r="F53" s="46"/>
@@ -1693,11 +1815,13 @@
       <x:c r="M53" s="46"/>
       <x:c r="N53" s="46"/>
       <x:c r="O53" s="58"/>
+      <x:c r="P53" s="58"/>
+      <x:c r="Q53" s="61"/>
     </x:row>
     <x:row r="54" ht="15" hidden="0" customHeight="1">
       <x:c r="A54" s="52"/>
       <x:c r="B54" s="46"/>
-      <x:c r="C54" s="61"/>
+      <x:c r="C54" s="64"/>
       <x:c r="D54" s="55"/>
       <x:c r="E54" s="46"/>
       <x:c r="F54" s="46"/>
@@ -1710,11 +1834,13 @@
       <x:c r="M54" s="46"/>
       <x:c r="N54" s="46"/>
       <x:c r="O54" s="58"/>
+      <x:c r="P54" s="58"/>
+      <x:c r="Q54" s="61"/>
     </x:row>
     <x:row r="55" ht="15" hidden="0" customHeight="1">
       <x:c r="A55" s="52"/>
       <x:c r="B55" s="46"/>
-      <x:c r="C55" s="61"/>
+      <x:c r="C55" s="64"/>
       <x:c r="D55" s="55"/>
       <x:c r="E55" s="46"/>
       <x:c r="F55" s="46"/>
@@ -1727,11 +1853,13 @@
       <x:c r="M55" s="46"/>
       <x:c r="N55" s="46"/>
       <x:c r="O55" s="58"/>
+      <x:c r="P55" s="58"/>
+      <x:c r="Q55" s="61"/>
     </x:row>
     <x:row r="56" ht="15" hidden="0" customHeight="1">
       <x:c r="A56" s="52"/>
       <x:c r="B56" s="46"/>
-      <x:c r="C56" s="61"/>
+      <x:c r="C56" s="64"/>
       <x:c r="D56" s="55"/>
       <x:c r="E56" s="46"/>
       <x:c r="F56" s="46"/>
@@ -1744,11 +1872,13 @@
       <x:c r="M56" s="46"/>
       <x:c r="N56" s="46"/>
       <x:c r="O56" s="58"/>
+      <x:c r="P56" s="58"/>
+      <x:c r="Q56" s="61"/>
     </x:row>
     <x:row r="57" ht="15" hidden="0" customHeight="1">
       <x:c r="A57" s="52"/>
       <x:c r="B57" s="46"/>
-      <x:c r="C57" s="61"/>
+      <x:c r="C57" s="64"/>
       <x:c r="D57" s="55"/>
       <x:c r="E57" s="46"/>
       <x:c r="F57" s="46"/>
@@ -1761,11 +1891,13 @@
       <x:c r="M57" s="46"/>
       <x:c r="N57" s="46"/>
       <x:c r="O57" s="58"/>
+      <x:c r="P57" s="58"/>
+      <x:c r="Q57" s="61"/>
     </x:row>
     <x:row r="58" ht="15" hidden="0" customHeight="1">
       <x:c r="A58" s="52"/>
       <x:c r="B58" s="46"/>
-      <x:c r="C58" s="61"/>
+      <x:c r="C58" s="64"/>
       <x:c r="D58" s="55"/>
       <x:c r="E58" s="46"/>
       <x:c r="F58" s="46"/>
@@ -1778,11 +1910,13 @@
       <x:c r="M58" s="46"/>
       <x:c r="N58" s="46"/>
       <x:c r="O58" s="58"/>
+      <x:c r="P58" s="58"/>
+      <x:c r="Q58" s="61"/>
     </x:row>
     <x:row r="59" ht="15" hidden="0" customHeight="1">
       <x:c r="A59" s="52"/>
       <x:c r="B59" s="46"/>
-      <x:c r="C59" s="61"/>
+      <x:c r="C59" s="64"/>
       <x:c r="D59" s="55"/>
       <x:c r="E59" s="46"/>
       <x:c r="F59" s="46"/>
@@ -1795,11 +1929,13 @@
       <x:c r="M59" s="46"/>
       <x:c r="N59" s="46"/>
       <x:c r="O59" s="58"/>
+      <x:c r="P59" s="58"/>
+      <x:c r="Q59" s="61"/>
     </x:row>
     <x:row r="60" ht="15" hidden="0" customHeight="1">
       <x:c r="A60" s="52"/>
       <x:c r="B60" s="46"/>
-      <x:c r="C60" s="61"/>
+      <x:c r="C60" s="64"/>
       <x:c r="D60" s="55"/>
       <x:c r="E60" s="46"/>
       <x:c r="F60" s="46"/>
@@ -1812,11 +1948,13 @@
       <x:c r="M60" s="46"/>
       <x:c r="N60" s="46"/>
       <x:c r="O60" s="58"/>
+      <x:c r="P60" s="58"/>
+      <x:c r="Q60" s="61"/>
     </x:row>
     <x:row r="61" ht="15" hidden="0" customHeight="1">
       <x:c r="A61" s="52"/>
       <x:c r="B61" s="46"/>
-      <x:c r="C61" s="61"/>
+      <x:c r="C61" s="64"/>
       <x:c r="D61" s="55"/>
       <x:c r="E61" s="46"/>
       <x:c r="F61" s="46"/>
@@ -1829,11 +1967,13 @@
       <x:c r="M61" s="46"/>
       <x:c r="N61" s="46"/>
       <x:c r="O61" s="58"/>
+      <x:c r="P61" s="58"/>
+      <x:c r="Q61" s="61"/>
     </x:row>
     <x:row r="62" ht="15" hidden="0" customHeight="1">
       <x:c r="A62" s="52"/>
       <x:c r="B62" s="46"/>
-      <x:c r="C62" s="61"/>
+      <x:c r="C62" s="64"/>
       <x:c r="D62" s="55"/>
       <x:c r="E62" s="46"/>
       <x:c r="F62" s="46"/>
@@ -1846,11 +1986,13 @@
       <x:c r="M62" s="46"/>
       <x:c r="N62" s="46"/>
       <x:c r="O62" s="58"/>
+      <x:c r="P62" s="58"/>
+      <x:c r="Q62" s="61"/>
     </x:row>
     <x:row r="63" ht="15" hidden="0" customHeight="1">
       <x:c r="A63" s="52"/>
       <x:c r="B63" s="46"/>
-      <x:c r="C63" s="61"/>
+      <x:c r="C63" s="64"/>
       <x:c r="D63" s="55"/>
       <x:c r="E63" s="46"/>
       <x:c r="F63" s="46"/>
@@ -1863,11 +2005,13 @@
       <x:c r="M63" s="46"/>
       <x:c r="N63" s="46"/>
       <x:c r="O63" s="58"/>
+      <x:c r="P63" s="58"/>
+      <x:c r="Q63" s="61"/>
     </x:row>
     <x:row r="64" ht="15" hidden="0" customHeight="1">
       <x:c r="A64" s="52"/>
       <x:c r="B64" s="46"/>
-      <x:c r="C64" s="61"/>
+      <x:c r="C64" s="64"/>
       <x:c r="D64" s="55"/>
       <x:c r="E64" s="46"/>
       <x:c r="F64" s="46"/>
@@ -1880,11 +2024,13 @@
       <x:c r="M64" s="46"/>
       <x:c r="N64" s="46"/>
       <x:c r="O64" s="58"/>
+      <x:c r="P64" s="58"/>
+      <x:c r="Q64" s="61"/>
     </x:row>
     <x:row r="65" ht="15" hidden="0" customHeight="1">
       <x:c r="A65" s="52"/>
       <x:c r="B65" s="46"/>
-      <x:c r="C65" s="61"/>
+      <x:c r="C65" s="64"/>
       <x:c r="D65" s="55"/>
       <x:c r="E65" s="46"/>
       <x:c r="F65" s="46"/>
@@ -1897,11 +2043,13 @@
       <x:c r="M65" s="46"/>
       <x:c r="N65" s="46"/>
       <x:c r="O65" s="58"/>
+      <x:c r="P65" s="58"/>
+      <x:c r="Q65" s="61"/>
     </x:row>
     <x:row r="66" ht="15" hidden="0" customHeight="1">
       <x:c r="A66" s="52"/>
       <x:c r="B66" s="46"/>
-      <x:c r="C66" s="61"/>
+      <x:c r="C66" s="64"/>
       <x:c r="D66" s="55"/>
       <x:c r="E66" s="46"/>
       <x:c r="F66" s="46"/>
@@ -1914,11 +2062,13 @@
       <x:c r="M66" s="46"/>
       <x:c r="N66" s="46"/>
       <x:c r="O66" s="58"/>
+      <x:c r="P66" s="58"/>
+      <x:c r="Q66" s="61"/>
     </x:row>
     <x:row r="67" ht="15" hidden="0" customHeight="1">
       <x:c r="A67" s="52"/>
       <x:c r="B67" s="46"/>
-      <x:c r="C67" s="61"/>
+      <x:c r="C67" s="64"/>
       <x:c r="D67" s="55"/>
       <x:c r="E67" s="46"/>
       <x:c r="F67" s="46"/>
@@ -1931,11 +2081,13 @@
       <x:c r="M67" s="46"/>
       <x:c r="N67" s="46"/>
       <x:c r="O67" s="58"/>
+      <x:c r="P67" s="58"/>
+      <x:c r="Q67" s="61"/>
     </x:row>
     <x:row r="68" ht="15" hidden="0" customHeight="1">
       <x:c r="A68" s="52"/>
       <x:c r="B68" s="46"/>
-      <x:c r="C68" s="61"/>
+      <x:c r="C68" s="64"/>
       <x:c r="D68" s="55"/>
       <x:c r="E68" s="46"/>
       <x:c r="F68" s="46"/>
@@ -1948,11 +2100,13 @@
       <x:c r="M68" s="46"/>
       <x:c r="N68" s="46"/>
       <x:c r="O68" s="58"/>
+      <x:c r="P68" s="58"/>
+      <x:c r="Q68" s="61"/>
     </x:row>
     <x:row r="69" ht="15" hidden="0" customHeight="1">
       <x:c r="A69" s="52"/>
       <x:c r="B69" s="46"/>
-      <x:c r="C69" s="61"/>
+      <x:c r="C69" s="64"/>
       <x:c r="D69" s="55"/>
       <x:c r="E69" s="46"/>
       <x:c r="F69" s="46"/>
@@ -1965,11 +2119,13 @@
       <x:c r="M69" s="46"/>
       <x:c r="N69" s="46"/>
       <x:c r="O69" s="58"/>
+      <x:c r="P69" s="58"/>
+      <x:c r="Q69" s="61"/>
     </x:row>
     <x:row r="70" ht="15" hidden="0" customHeight="1">
       <x:c r="A70" s="52"/>
       <x:c r="B70" s="46"/>
-      <x:c r="C70" s="61"/>
+      <x:c r="C70" s="64"/>
       <x:c r="D70" s="55"/>
       <x:c r="E70" s="46"/>
       <x:c r="F70" s="46"/>
@@ -1982,11 +2138,13 @@
       <x:c r="M70" s="46"/>
       <x:c r="N70" s="46"/>
       <x:c r="O70" s="58"/>
+      <x:c r="P70" s="58"/>
+      <x:c r="Q70" s="61"/>
     </x:row>
     <x:row r="71" ht="15" hidden="0" customHeight="1">
       <x:c r="A71" s="52"/>
       <x:c r="B71" s="46"/>
-      <x:c r="C71" s="61"/>
+      <x:c r="C71" s="64"/>
       <x:c r="D71" s="55"/>
       <x:c r="E71" s="46"/>
       <x:c r="F71" s="46"/>
@@ -1999,11 +2157,13 @@
       <x:c r="M71" s="46"/>
       <x:c r="N71" s="46"/>
       <x:c r="O71" s="58"/>
+      <x:c r="P71" s="58"/>
+      <x:c r="Q71" s="61"/>
     </x:row>
     <x:row r="72" ht="15" hidden="0" customHeight="1">
       <x:c r="A72" s="52"/>
       <x:c r="B72" s="46"/>
-      <x:c r="C72" s="61"/>
+      <x:c r="C72" s="64"/>
       <x:c r="D72" s="55"/>
       <x:c r="E72" s="46"/>
       <x:c r="F72" s="46"/>
@@ -2016,11 +2176,13 @@
       <x:c r="M72" s="46"/>
       <x:c r="N72" s="46"/>
       <x:c r="O72" s="58"/>
+      <x:c r="P72" s="58"/>
+      <x:c r="Q72" s="61"/>
     </x:row>
     <x:row r="73" ht="15" hidden="0" customHeight="1">
       <x:c r="A73" s="52"/>
       <x:c r="B73" s="46"/>
-      <x:c r="C73" s="61"/>
+      <x:c r="C73" s="64"/>
       <x:c r="D73" s="55"/>
       <x:c r="E73" s="46"/>
       <x:c r="F73" s="46"/>
@@ -2033,11 +2195,13 @@
       <x:c r="M73" s="46"/>
       <x:c r="N73" s="46"/>
       <x:c r="O73" s="58"/>
+      <x:c r="P73" s="58"/>
+      <x:c r="Q73" s="61"/>
     </x:row>
     <x:row r="74" ht="15" hidden="0" customHeight="1">
       <x:c r="A74" s="52"/>
       <x:c r="B74" s="46"/>
-      <x:c r="C74" s="61"/>
+      <x:c r="C74" s="64"/>
       <x:c r="D74" s="55"/>
       <x:c r="E74" s="46"/>
       <x:c r="F74" s="46"/>
@@ -2050,11 +2214,13 @@
       <x:c r="M74" s="46"/>
       <x:c r="N74" s="46"/>
       <x:c r="O74" s="58"/>
+      <x:c r="P74" s="58"/>
+      <x:c r="Q74" s="61"/>
     </x:row>
     <x:row r="75" ht="15" hidden="0" customHeight="1">
       <x:c r="A75" s="52"/>
       <x:c r="B75" s="46"/>
-      <x:c r="C75" s="61"/>
+      <x:c r="C75" s="64"/>
       <x:c r="D75" s="55"/>
       <x:c r="E75" s="46"/>
       <x:c r="F75" s="46"/>
@@ -2067,11 +2233,13 @@
       <x:c r="M75" s="46"/>
       <x:c r="N75" s="46"/>
       <x:c r="O75" s="58"/>
+      <x:c r="P75" s="58"/>
+      <x:c r="Q75" s="61"/>
     </x:row>
     <x:row r="76" ht="15" hidden="0" customHeight="1">
       <x:c r="A76" s="52"/>
       <x:c r="B76" s="46"/>
-      <x:c r="C76" s="61"/>
+      <x:c r="C76" s="64"/>
       <x:c r="D76" s="55"/>
       <x:c r="E76" s="46"/>
       <x:c r="F76" s="46"/>
@@ -2084,11 +2252,13 @@
       <x:c r="M76" s="46"/>
       <x:c r="N76" s="46"/>
       <x:c r="O76" s="58"/>
+      <x:c r="P76" s="58"/>
+      <x:c r="Q76" s="61"/>
     </x:row>
     <x:row r="77" ht="15" hidden="0" customHeight="1">
       <x:c r="A77" s="52"/>
       <x:c r="B77" s="46"/>
-      <x:c r="C77" s="61"/>
+      <x:c r="C77" s="64"/>
       <x:c r="D77" s="55"/>
       <x:c r="E77" s="46"/>
       <x:c r="F77" s="46"/>
@@ -2101,11 +2271,13 @@
       <x:c r="M77" s="46"/>
       <x:c r="N77" s="46"/>
       <x:c r="O77" s="58"/>
+      <x:c r="P77" s="58"/>
+      <x:c r="Q77" s="61"/>
     </x:row>
     <x:row r="78" ht="15" hidden="0" customHeight="1">
       <x:c r="A78" s="52"/>
       <x:c r="B78" s="46"/>
-      <x:c r="C78" s="61"/>
+      <x:c r="C78" s="64"/>
       <x:c r="D78" s="55"/>
       <x:c r="E78" s="46"/>
       <x:c r="F78" s="46"/>
@@ -2118,11 +2290,13 @@
       <x:c r="M78" s="46"/>
       <x:c r="N78" s="46"/>
       <x:c r="O78" s="58"/>
+      <x:c r="P78" s="58"/>
+      <x:c r="Q78" s="61"/>
     </x:row>
     <x:row r="79" ht="15" hidden="0" customHeight="1">
       <x:c r="A79" s="52"/>
       <x:c r="B79" s="46"/>
-      <x:c r="C79" s="61"/>
+      <x:c r="C79" s="64"/>
       <x:c r="D79" s="55"/>
       <x:c r="E79" s="46"/>
       <x:c r="F79" s="46"/>
@@ -2135,11 +2309,13 @@
       <x:c r="M79" s="46"/>
       <x:c r="N79" s="46"/>
       <x:c r="O79" s="58"/>
+      <x:c r="P79" s="58"/>
+      <x:c r="Q79" s="61"/>
     </x:row>
     <x:row r="80" ht="15" hidden="0" customHeight="1">
       <x:c r="A80" s="52"/>
       <x:c r="B80" s="46"/>
-      <x:c r="C80" s="61"/>
+      <x:c r="C80" s="64"/>
       <x:c r="D80" s="55"/>
       <x:c r="E80" s="46"/>
       <x:c r="F80" s="46"/>
@@ -2152,11 +2328,13 @@
       <x:c r="M80" s="46"/>
       <x:c r="N80" s="46"/>
       <x:c r="O80" s="58"/>
+      <x:c r="P80" s="58"/>
+      <x:c r="Q80" s="61"/>
     </x:row>
     <x:row r="81" ht="15" hidden="0" customHeight="1">
       <x:c r="A81" s="52"/>
       <x:c r="B81" s="46"/>
-      <x:c r="C81" s="61"/>
+      <x:c r="C81" s="64"/>
       <x:c r="D81" s="55"/>
       <x:c r="E81" s="46"/>
       <x:c r="F81" s="46"/>
@@ -2169,11 +2347,13 @@
       <x:c r="M81" s="46"/>
       <x:c r="N81" s="46"/>
       <x:c r="O81" s="58"/>
+      <x:c r="P81" s="58"/>
+      <x:c r="Q81" s="61"/>
     </x:row>
     <x:row r="82" ht="15" hidden="0" customHeight="1">
       <x:c r="A82" s="52"/>
       <x:c r="B82" s="46"/>
-      <x:c r="C82" s="61"/>
+      <x:c r="C82" s="64"/>
       <x:c r="D82" s="55"/>
       <x:c r="E82" s="46"/>
       <x:c r="F82" s="46"/>
@@ -2186,11 +2366,13 @@
       <x:c r="M82" s="46"/>
       <x:c r="N82" s="46"/>
       <x:c r="O82" s="58"/>
+      <x:c r="P82" s="58"/>
+      <x:c r="Q82" s="61"/>
     </x:row>
     <x:row r="83" ht="15" hidden="0" customHeight="1">
       <x:c r="A83" s="52"/>
       <x:c r="B83" s="46"/>
-      <x:c r="C83" s="61"/>
+      <x:c r="C83" s="64"/>
       <x:c r="D83" s="55"/>
       <x:c r="E83" s="46"/>
       <x:c r="F83" s="46"/>
@@ -2203,11 +2385,13 @@
       <x:c r="M83" s="46"/>
       <x:c r="N83" s="46"/>
       <x:c r="O83" s="58"/>
+      <x:c r="P83" s="58"/>
+      <x:c r="Q83" s="61"/>
     </x:row>
     <x:row r="84" ht="15" hidden="0" customHeight="1">
       <x:c r="A84" s="52"/>
       <x:c r="B84" s="46"/>
-      <x:c r="C84" s="61"/>
+      <x:c r="C84" s="64"/>
       <x:c r="D84" s="55"/>
       <x:c r="E84" s="46"/>
       <x:c r="F84" s="46"/>
@@ -2220,11 +2404,13 @@
       <x:c r="M84" s="46"/>
       <x:c r="N84" s="46"/>
       <x:c r="O84" s="58"/>
+      <x:c r="P84" s="58"/>
+      <x:c r="Q84" s="61"/>
     </x:row>
     <x:row r="85" ht="15" hidden="0" customHeight="1">
       <x:c r="A85" s="52"/>
       <x:c r="B85" s="46"/>
-      <x:c r="C85" s="61"/>
+      <x:c r="C85" s="64"/>
       <x:c r="D85" s="55"/>
       <x:c r="E85" s="46"/>
       <x:c r="F85" s="46"/>
@@ -2237,11 +2423,13 @@
       <x:c r="M85" s="46"/>
       <x:c r="N85" s="46"/>
       <x:c r="O85" s="58"/>
+      <x:c r="P85" s="58"/>
+      <x:c r="Q85" s="61"/>
     </x:row>
     <x:row r="86" ht="15" hidden="0" customHeight="1">
       <x:c r="A86" s="52"/>
       <x:c r="B86" s="46"/>
-      <x:c r="C86" s="61"/>
+      <x:c r="C86" s="64"/>
       <x:c r="D86" s="55"/>
       <x:c r="E86" s="46"/>
       <x:c r="F86" s="46"/>
@@ -2254,11 +2442,13 @@
       <x:c r="M86" s="46"/>
       <x:c r="N86" s="46"/>
       <x:c r="O86" s="58"/>
+      <x:c r="P86" s="58"/>
+      <x:c r="Q86" s="61"/>
     </x:row>
     <x:row r="87" ht="15" hidden="0" customHeight="1">
       <x:c r="A87" s="52"/>
       <x:c r="B87" s="46"/>
-      <x:c r="C87" s="61"/>
+      <x:c r="C87" s="64"/>
       <x:c r="D87" s="55"/>
       <x:c r="E87" s="46"/>
       <x:c r="F87" s="46"/>
@@ -2271,11 +2461,13 @@
       <x:c r="M87" s="46"/>
       <x:c r="N87" s="46"/>
       <x:c r="O87" s="58"/>
+      <x:c r="P87" s="58"/>
+      <x:c r="Q87" s="61"/>
     </x:row>
     <x:row r="88" ht="15" hidden="0" customHeight="1">
       <x:c r="A88" s="52"/>
       <x:c r="B88" s="46"/>
-      <x:c r="C88" s="61"/>
+      <x:c r="C88" s="64"/>
       <x:c r="D88" s="55"/>
       <x:c r="E88" s="46"/>
       <x:c r="F88" s="46"/>
@@ -2288,11 +2480,13 @@
       <x:c r="M88" s="46"/>
       <x:c r="N88" s="46"/>
       <x:c r="O88" s="58"/>
+      <x:c r="P88" s="58"/>
+      <x:c r="Q88" s="61"/>
     </x:row>
     <x:row r="89" ht="15" hidden="0" customHeight="1">
       <x:c r="A89" s="52"/>
       <x:c r="B89" s="46"/>
-      <x:c r="C89" s="61"/>
+      <x:c r="C89" s="64"/>
       <x:c r="D89" s="55"/>
       <x:c r="E89" s="46"/>
       <x:c r="F89" s="46"/>
@@ -2305,11 +2499,13 @@
       <x:c r="M89" s="46"/>
       <x:c r="N89" s="46"/>
       <x:c r="O89" s="58"/>
+      <x:c r="P89" s="58"/>
+      <x:c r="Q89" s="61"/>
     </x:row>
     <x:row r="90" ht="15" hidden="0" customHeight="1">
       <x:c r="A90" s="52"/>
       <x:c r="B90" s="46"/>
-      <x:c r="C90" s="61"/>
+      <x:c r="C90" s="64"/>
       <x:c r="D90" s="55"/>
       <x:c r="E90" s="46"/>
       <x:c r="F90" s="46"/>
@@ -2322,11 +2518,13 @@
       <x:c r="M90" s="46"/>
       <x:c r="N90" s="46"/>
       <x:c r="O90" s="58"/>
+      <x:c r="P90" s="58"/>
+      <x:c r="Q90" s="61"/>
     </x:row>
     <x:row r="91" ht="15" hidden="0" customHeight="1">
       <x:c r="A91" s="52"/>
       <x:c r="B91" s="46"/>
-      <x:c r="C91" s="61"/>
+      <x:c r="C91" s="64"/>
       <x:c r="D91" s="55"/>
       <x:c r="E91" s="46"/>
       <x:c r="F91" s="46"/>
@@ -2339,11 +2537,13 @@
       <x:c r="M91" s="46"/>
       <x:c r="N91" s="46"/>
       <x:c r="O91" s="58"/>
+      <x:c r="P91" s="58"/>
+      <x:c r="Q91" s="61"/>
     </x:row>
     <x:row r="92" ht="15" hidden="0" customHeight="1">
       <x:c r="A92" s="52"/>
       <x:c r="B92" s="46"/>
-      <x:c r="C92" s="61"/>
+      <x:c r="C92" s="64"/>
       <x:c r="D92" s="55"/>
       <x:c r="E92" s="46"/>
       <x:c r="F92" s="46"/>
@@ -2356,11 +2556,13 @@
       <x:c r="M92" s="46"/>
       <x:c r="N92" s="46"/>
       <x:c r="O92" s="58"/>
+      <x:c r="P92" s="58"/>
+      <x:c r="Q92" s="61"/>
     </x:row>
     <x:row r="93" ht="15" hidden="0" customHeight="1">
       <x:c r="A93" s="52"/>
       <x:c r="B93" s="46"/>
-      <x:c r="C93" s="61"/>
+      <x:c r="C93" s="64"/>
       <x:c r="D93" s="55"/>
       <x:c r="E93" s="46"/>
       <x:c r="F93" s="46"/>
@@ -2373,11 +2575,13 @@
       <x:c r="M93" s="46"/>
       <x:c r="N93" s="46"/>
       <x:c r="O93" s="58"/>
+      <x:c r="P93" s="58"/>
+      <x:c r="Q93" s="61"/>
     </x:row>
     <x:row r="94" ht="15" hidden="0" customHeight="1">
       <x:c r="A94" s="52"/>
       <x:c r="B94" s="46"/>
-      <x:c r="C94" s="61"/>
+      <x:c r="C94" s="64"/>
       <x:c r="D94" s="55"/>
       <x:c r="E94" s="46"/>
       <x:c r="F94" s="46"/>
@@ -2390,11 +2594,13 @@
       <x:c r="M94" s="46"/>
       <x:c r="N94" s="46"/>
       <x:c r="O94" s="58"/>
+      <x:c r="P94" s="58"/>
+      <x:c r="Q94" s="61"/>
     </x:row>
     <x:row r="95" ht="15" hidden="0" customHeight="1">
       <x:c r="A95" s="52"/>
       <x:c r="B95" s="46"/>
-      <x:c r="C95" s="61"/>
+      <x:c r="C95" s="64"/>
       <x:c r="D95" s="55"/>
       <x:c r="E95" s="46"/>
       <x:c r="F95" s="46"/>
@@ -2407,11 +2613,13 @@
       <x:c r="M95" s="46"/>
       <x:c r="N95" s="46"/>
       <x:c r="O95" s="58"/>
+      <x:c r="P95" s="58"/>
+      <x:c r="Q95" s="61"/>
     </x:row>
     <x:row r="96" ht="15" hidden="0" customHeight="1">
       <x:c r="A96" s="52"/>
       <x:c r="B96" s="46"/>
-      <x:c r="C96" s="61"/>
+      <x:c r="C96" s="64"/>
       <x:c r="D96" s="55"/>
       <x:c r="E96" s="46"/>
       <x:c r="F96" s="46"/>
@@ -2424,11 +2632,13 @@
       <x:c r="M96" s="46"/>
       <x:c r="N96" s="46"/>
       <x:c r="O96" s="58"/>
+      <x:c r="P96" s="58"/>
+      <x:c r="Q96" s="61"/>
     </x:row>
     <x:row r="97" ht="15" hidden="0" customHeight="1">
       <x:c r="A97" s="52"/>
       <x:c r="B97" s="46"/>
-      <x:c r="C97" s="61"/>
+      <x:c r="C97" s="64"/>
       <x:c r="D97" s="55"/>
       <x:c r="E97" s="46"/>
       <x:c r="F97" s="46"/>
@@ -2441,11 +2651,13 @@
       <x:c r="M97" s="46"/>
       <x:c r="N97" s="46"/>
       <x:c r="O97" s="58"/>
+      <x:c r="P97" s="58"/>
+      <x:c r="Q97" s="61"/>
     </x:row>
     <x:row r="98" ht="15" hidden="0" customHeight="1">
       <x:c r="A98" s="52"/>
       <x:c r="B98" s="46"/>
-      <x:c r="C98" s="61"/>
+      <x:c r="C98" s="64"/>
       <x:c r="D98" s="55"/>
       <x:c r="E98" s="46"/>
       <x:c r="F98" s="46"/>
@@ -2458,11 +2670,13 @@
       <x:c r="M98" s="46"/>
       <x:c r="N98" s="46"/>
       <x:c r="O98" s="58"/>
+      <x:c r="P98" s="58"/>
+      <x:c r="Q98" s="61"/>
     </x:row>
     <x:row r="99" ht="15" hidden="0" customHeight="1">
       <x:c r="A99" s="52"/>
       <x:c r="B99" s="46"/>
-      <x:c r="C99" s="61"/>
+      <x:c r="C99" s="64"/>
       <x:c r="D99" s="55"/>
       <x:c r="E99" s="46"/>
       <x:c r="F99" s="46"/>
@@ -2475,11 +2689,13 @@
       <x:c r="M99" s="46"/>
       <x:c r="N99" s="46"/>
       <x:c r="O99" s="58"/>
+      <x:c r="P99" s="58"/>
+      <x:c r="Q99" s="61"/>
     </x:row>
     <x:row r="100" ht="15" hidden="0" customHeight="1">
       <x:c r="A100" s="52"/>
       <x:c r="B100" s="46"/>
-      <x:c r="C100" s="61"/>
+      <x:c r="C100" s="64"/>
       <x:c r="D100" s="55"/>
       <x:c r="E100" s="46"/>
       <x:c r="F100" s="46"/>
@@ -2492,11 +2708,13 @@
       <x:c r="M100" s="46"/>
       <x:c r="N100" s="46"/>
       <x:c r="O100" s="58"/>
+      <x:c r="P100" s="58"/>
+      <x:c r="Q100" s="61"/>
     </x:row>
     <x:row r="101" ht="15" hidden="0" customHeight="1">
       <x:c r="A101" s="52"/>
       <x:c r="B101" s="46"/>
-      <x:c r="C101" s="61"/>
+      <x:c r="C101" s="64"/>
       <x:c r="D101" s="55"/>
       <x:c r="E101" s="46"/>
       <x:c r="F101" s="46"/>
@@ -2509,11 +2727,13 @@
       <x:c r="M101" s="46"/>
       <x:c r="N101" s="46"/>
       <x:c r="O101" s="58"/>
+      <x:c r="P101" s="58"/>
+      <x:c r="Q101" s="61"/>
     </x:row>
     <x:row r="102" ht="15" hidden="0" customHeight="1">
       <x:c r="A102" s="52"/>
       <x:c r="B102" s="46"/>
-      <x:c r="C102" s="61"/>
+      <x:c r="C102" s="64"/>
       <x:c r="D102" s="55"/>
       <x:c r="E102" s="46"/>
       <x:c r="F102" s="46"/>
@@ -2526,11 +2746,13 @@
       <x:c r="M102" s="46"/>
       <x:c r="N102" s="46"/>
       <x:c r="O102" s="58"/>
+      <x:c r="P102" s="58"/>
+      <x:c r="Q102" s="61"/>
     </x:row>
     <x:row r="103" ht="15" hidden="0" customHeight="1">
       <x:c r="A103" s="52"/>
       <x:c r="B103" s="46"/>
-      <x:c r="C103" s="61"/>
+      <x:c r="C103" s="64"/>
       <x:c r="D103" s="55"/>
       <x:c r="E103" s="46"/>
       <x:c r="F103" s="46"/>
@@ -2543,11 +2765,13 @@
       <x:c r="M103" s="46"/>
       <x:c r="N103" s="46"/>
       <x:c r="O103" s="58"/>
+      <x:c r="P103" s="58"/>
+      <x:c r="Q103" s="61"/>
     </x:row>
     <x:row r="104" ht="15" hidden="0" customHeight="1">
       <x:c r="A104" s="52"/>
       <x:c r="B104" s="46"/>
-      <x:c r="C104" s="61"/>
+      <x:c r="C104" s="64"/>
       <x:c r="D104" s="55"/>
       <x:c r="E104" s="46"/>
       <x:c r="F104" s="46"/>
@@ -2560,11 +2784,13 @@
       <x:c r="M104" s="46"/>
       <x:c r="N104" s="46"/>
       <x:c r="O104" s="58"/>
+      <x:c r="P104" s="58"/>
+      <x:c r="Q104" s="61"/>
     </x:row>
     <x:row r="105" ht="15" hidden="0" customHeight="1">
       <x:c r="A105" s="52"/>
       <x:c r="B105" s="46"/>
-      <x:c r="C105" s="61"/>
+      <x:c r="C105" s="64"/>
       <x:c r="D105" s="55"/>
       <x:c r="E105" s="46"/>
       <x:c r="F105" s="46"/>
@@ -2577,11 +2803,13 @@
       <x:c r="M105" s="46"/>
       <x:c r="N105" s="46"/>
       <x:c r="O105" s="58"/>
+      <x:c r="P105" s="58"/>
+      <x:c r="Q105" s="61"/>
     </x:row>
     <x:row r="106" ht="15" hidden="0" customHeight="1">
       <x:c r="A106" s="52"/>
       <x:c r="B106" s="46"/>
-      <x:c r="C106" s="61"/>
+      <x:c r="C106" s="64"/>
       <x:c r="D106" s="55"/>
       <x:c r="E106" s="46"/>
       <x:c r="F106" s="46"/>
@@ -2594,11 +2822,13 @@
       <x:c r="M106" s="46"/>
       <x:c r="N106" s="46"/>
       <x:c r="O106" s="58"/>
+      <x:c r="P106" s="58"/>
+      <x:c r="Q106" s="61"/>
     </x:row>
     <x:row r="107" ht="15" hidden="0" customHeight="1">
       <x:c r="A107" s="52"/>
       <x:c r="B107" s="46"/>
-      <x:c r="C107" s="61"/>
+      <x:c r="C107" s="64"/>
       <x:c r="D107" s="55"/>
       <x:c r="E107" s="46"/>
       <x:c r="F107" s="46"/>
@@ -2611,11 +2841,13 @@
       <x:c r="M107" s="46"/>
       <x:c r="N107" s="46"/>
       <x:c r="O107" s="58"/>
+      <x:c r="P107" s="58"/>
+      <x:c r="Q107" s="61"/>
     </x:row>
     <x:row r="108" ht="15" hidden="0" customHeight="1">
       <x:c r="A108" s="52"/>
       <x:c r="B108" s="46"/>
-      <x:c r="C108" s="61"/>
+      <x:c r="C108" s="64"/>
       <x:c r="D108" s="55"/>
       <x:c r="E108" s="46"/>
       <x:c r="F108" s="46"/>
@@ -2628,11 +2860,13 @@
       <x:c r="M108" s="46"/>
       <x:c r="N108" s="46"/>
       <x:c r="O108" s="58"/>
+      <x:c r="P108" s="58"/>
+      <x:c r="Q108" s="61"/>
     </x:row>
     <x:row r="109" ht="15" hidden="0" customHeight="1">
       <x:c r="A109" s="52"/>
       <x:c r="B109" s="46"/>
-      <x:c r="C109" s="61"/>
+      <x:c r="C109" s="64"/>
       <x:c r="D109" s="55"/>
       <x:c r="E109" s="46"/>
       <x:c r="F109" s="46"/>
@@ -2645,11 +2879,13 @@
       <x:c r="M109" s="46"/>
       <x:c r="N109" s="46"/>
       <x:c r="O109" s="58"/>
+      <x:c r="P109" s="58"/>
+      <x:c r="Q109" s="61"/>
     </x:row>
     <x:row r="110" ht="15" hidden="0" customHeight="1">
       <x:c r="A110" s="52"/>
       <x:c r="B110" s="46"/>
-      <x:c r="C110" s="61"/>
+      <x:c r="C110" s="64"/>
       <x:c r="D110" s="55"/>
       <x:c r="E110" s="46"/>
       <x:c r="F110" s="46"/>
@@ -2662,11 +2898,13 @@
       <x:c r="M110" s="46"/>
       <x:c r="N110" s="46"/>
       <x:c r="O110" s="58"/>
+      <x:c r="P110" s="58"/>
+      <x:c r="Q110" s="61"/>
     </x:row>
     <x:row r="111" ht="15" hidden="0" customHeight="1">
       <x:c r="A111" s="52"/>
       <x:c r="B111" s="46"/>
-      <x:c r="C111" s="61"/>
+      <x:c r="C111" s="64"/>
       <x:c r="D111" s="55"/>
       <x:c r="E111" s="46"/>
       <x:c r="F111" s="46"/>
@@ -2679,11 +2917,13 @@
       <x:c r="M111" s="46"/>
       <x:c r="N111" s="46"/>
       <x:c r="O111" s="58"/>
+      <x:c r="P111" s="58"/>
+      <x:c r="Q111" s="61"/>
     </x:row>
     <x:row r="112" ht="15" hidden="0" customHeight="1">
       <x:c r="A112" s="52"/>
       <x:c r="B112" s="46"/>
-      <x:c r="C112" s="61"/>
+      <x:c r="C112" s="64"/>
       <x:c r="D112" s="55"/>
       <x:c r="E112" s="46"/>
       <x:c r="F112" s="46"/>
@@ -2696,11 +2936,13 @@
       <x:c r="M112" s="46"/>
       <x:c r="N112" s="46"/>
       <x:c r="O112" s="58"/>
+      <x:c r="P112" s="58"/>
+      <x:c r="Q112" s="61"/>
     </x:row>
     <x:row r="113" ht="15" hidden="0" customHeight="1">
       <x:c r="A113" s="52"/>
       <x:c r="B113" s="46"/>
-      <x:c r="C113" s="61"/>
+      <x:c r="C113" s="64"/>
       <x:c r="D113" s="55"/>
       <x:c r="E113" s="46"/>
       <x:c r="F113" s="46"/>
@@ -2713,11 +2955,13 @@
       <x:c r="M113" s="46"/>
       <x:c r="N113" s="46"/>
       <x:c r="O113" s="58"/>
+      <x:c r="P113" s="58"/>
+      <x:c r="Q113" s="61"/>
     </x:row>
     <x:row r="114" ht="15" hidden="0" customHeight="1">
       <x:c r="A114" s="52"/>
       <x:c r="B114" s="46"/>
-      <x:c r="C114" s="61"/>
+      <x:c r="C114" s="64"/>
       <x:c r="D114" s="55"/>
       <x:c r="E114" s="46"/>
       <x:c r="F114" s="46"/>
@@ -2730,11 +2974,13 @@
       <x:c r="M114" s="46"/>
       <x:c r="N114" s="46"/>
       <x:c r="O114" s="58"/>
+      <x:c r="P114" s="58"/>
+      <x:c r="Q114" s="61"/>
     </x:row>
     <x:row r="115" ht="15" hidden="0" customHeight="1">
       <x:c r="A115" s="52"/>
       <x:c r="B115" s="46"/>
-      <x:c r="C115" s="61"/>
+      <x:c r="C115" s="64"/>
       <x:c r="D115" s="55"/>
       <x:c r="E115" s="46"/>
       <x:c r="F115" s="46"/>
@@ -2747,11 +2993,13 @@
       <x:c r="M115" s="46"/>
       <x:c r="N115" s="46"/>
       <x:c r="O115" s="58"/>
+      <x:c r="P115" s="58"/>
+      <x:c r="Q115" s="61"/>
     </x:row>
     <x:row r="116" ht="15" hidden="0" customHeight="1">
       <x:c r="A116" s="52"/>
       <x:c r="B116" s="46"/>
-      <x:c r="C116" s="61"/>
+      <x:c r="C116" s="64"/>
       <x:c r="D116" s="55"/>
       <x:c r="E116" s="46"/>
       <x:c r="F116" s="46"/>
@@ -2764,11 +3012,13 @@
       <x:c r="M116" s="46"/>
       <x:c r="N116" s="46"/>
       <x:c r="O116" s="58"/>
+      <x:c r="P116" s="58"/>
+      <x:c r="Q116" s="61"/>
     </x:row>
     <x:row r="117" ht="15" hidden="0" customHeight="1">
       <x:c r="A117" s="52"/>
       <x:c r="B117" s="46"/>
-      <x:c r="C117" s="61"/>
+      <x:c r="C117" s="64"/>
       <x:c r="D117" s="55"/>
       <x:c r="E117" s="46"/>
       <x:c r="F117" s="46"/>
@@ -2781,11 +3031,13 @@
       <x:c r="M117" s="46"/>
       <x:c r="N117" s="46"/>
       <x:c r="O117" s="58"/>
+      <x:c r="P117" s="58"/>
+      <x:c r="Q117" s="61"/>
     </x:row>
     <x:row r="118" ht="15" hidden="0" customHeight="1">
       <x:c r="A118" s="52"/>
       <x:c r="B118" s="46"/>
-      <x:c r="C118" s="61"/>
+      <x:c r="C118" s="64"/>
       <x:c r="D118" s="55"/>
       <x:c r="E118" s="46"/>
       <x:c r="F118" s="46"/>
@@ -2798,11 +3050,13 @@
       <x:c r="M118" s="46"/>
       <x:c r="N118" s="46"/>
       <x:c r="O118" s="58"/>
+      <x:c r="P118" s="58"/>
+      <x:c r="Q118" s="61"/>
     </x:row>
     <x:row r="119" ht="15" hidden="0" customHeight="1">
       <x:c r="A119" s="52"/>
       <x:c r="B119" s="46"/>
-      <x:c r="C119" s="61"/>
+      <x:c r="C119" s="64"/>
       <x:c r="D119" s="55"/>
       <x:c r="E119" s="46"/>
       <x:c r="F119" s="46"/>
@@ -2815,11 +3069,13 @@
       <x:c r="M119" s="46"/>
       <x:c r="N119" s="46"/>
       <x:c r="O119" s="58"/>
+      <x:c r="P119" s="58"/>
+      <x:c r="Q119" s="61"/>
     </x:row>
     <x:row r="120" ht="15" hidden="0" customHeight="1">
       <x:c r="A120" s="52"/>
       <x:c r="B120" s="46"/>
-      <x:c r="C120" s="61"/>
+      <x:c r="C120" s="64"/>
       <x:c r="D120" s="55"/>
       <x:c r="E120" s="46"/>
       <x:c r="F120" s="46"/>
@@ -2832,11 +3088,13 @@
       <x:c r="M120" s="46"/>
       <x:c r="N120" s="46"/>
       <x:c r="O120" s="58"/>
+      <x:c r="P120" s="58"/>
+      <x:c r="Q120" s="61"/>
     </x:row>
     <x:row r="121" ht="15" hidden="0" customHeight="1">
       <x:c r="A121" s="52"/>
       <x:c r="B121" s="46"/>
-      <x:c r="C121" s="61"/>
+      <x:c r="C121" s="64"/>
       <x:c r="D121" s="55"/>
       <x:c r="E121" s="46"/>
       <x:c r="F121" s="46"/>
@@ -2849,11 +3107,13 @@
       <x:c r="M121" s="46"/>
       <x:c r="N121" s="46"/>
       <x:c r="O121" s="58"/>
+      <x:c r="P121" s="58"/>
+      <x:c r="Q121" s="61"/>
     </x:row>
     <x:row r="122" ht="15" hidden="0" customHeight="1">
       <x:c r="A122" s="52"/>
       <x:c r="B122" s="46"/>
-      <x:c r="C122" s="61"/>
+      <x:c r="C122" s="64"/>
       <x:c r="D122" s="55"/>
       <x:c r="E122" s="46"/>
       <x:c r="F122" s="46"/>
@@ -2866,11 +3126,13 @@
       <x:c r="M122" s="46"/>
       <x:c r="N122" s="46"/>
       <x:c r="O122" s="58"/>
+      <x:c r="P122" s="58"/>
+      <x:c r="Q122" s="61"/>
     </x:row>
     <x:row r="123" ht="15" hidden="0" customHeight="1">
       <x:c r="A123" s="52"/>
       <x:c r="B123" s="46"/>
-      <x:c r="C123" s="61"/>
+      <x:c r="C123" s="64"/>
       <x:c r="D123" s="55"/>
       <x:c r="E123" s="46"/>
       <x:c r="F123" s="46"/>
@@ -2883,11 +3145,13 @@
       <x:c r="M123" s="46"/>
       <x:c r="N123" s="46"/>
       <x:c r="O123" s="58"/>
+      <x:c r="P123" s="58"/>
+      <x:c r="Q123" s="61"/>
     </x:row>
     <x:row r="124" ht="15" hidden="0" customHeight="1">
       <x:c r="A124" s="52"/>
       <x:c r="B124" s="46"/>
-      <x:c r="C124" s="61"/>
+      <x:c r="C124" s="64"/>
       <x:c r="D124" s="55"/>
       <x:c r="E124" s="46"/>
       <x:c r="F124" s="46"/>
@@ -2900,11 +3164,13 @@
       <x:c r="M124" s="46"/>
       <x:c r="N124" s="46"/>
       <x:c r="O124" s="58"/>
+      <x:c r="P124" s="58"/>
+      <x:c r="Q124" s="61"/>
     </x:row>
     <x:row r="125" ht="15" hidden="0" customHeight="1">
       <x:c r="A125" s="52"/>
       <x:c r="B125" s="46"/>
-      <x:c r="C125" s="61"/>
+      <x:c r="C125" s="64"/>
       <x:c r="D125" s="55"/>
       <x:c r="E125" s="46"/>
       <x:c r="F125" s="46"/>
@@ -2917,11 +3183,13 @@
       <x:c r="M125" s="46"/>
       <x:c r="N125" s="46"/>
       <x:c r="O125" s="58"/>
+      <x:c r="P125" s="58"/>
+      <x:c r="Q125" s="61"/>
     </x:row>
     <x:row r="126" ht="15" hidden="0" customHeight="1">
       <x:c r="A126" s="52"/>
       <x:c r="B126" s="46"/>
-      <x:c r="C126" s="61"/>
+      <x:c r="C126" s="64"/>
       <x:c r="D126" s="55"/>
       <x:c r="E126" s="46"/>
       <x:c r="F126" s="46"/>
@@ -2934,11 +3202,13 @@
       <x:c r="M126" s="46"/>
       <x:c r="N126" s="46"/>
       <x:c r="O126" s="58"/>
+      <x:c r="P126" s="58"/>
+      <x:c r="Q126" s="61"/>
     </x:row>
     <x:row r="127" ht="15" hidden="0" customHeight="1">
       <x:c r="A127" s="52"/>
       <x:c r="B127" s="46"/>
-      <x:c r="C127" s="61"/>
+      <x:c r="C127" s="64"/>
       <x:c r="D127" s="55"/>
       <x:c r="E127" s="46"/>
       <x:c r="F127" s="46"/>
@@ -2951,11 +3221,13 @@
       <x:c r="M127" s="46"/>
       <x:c r="N127" s="46"/>
       <x:c r="O127" s="58"/>
+      <x:c r="P127" s="58"/>
+      <x:c r="Q127" s="61"/>
     </x:row>
     <x:row r="128" ht="15" hidden="0" customHeight="1">
       <x:c r="A128" s="52"/>
       <x:c r="B128" s="46"/>
-      <x:c r="C128" s="61"/>
+      <x:c r="C128" s="64"/>
       <x:c r="D128" s="55"/>
       <x:c r="E128" s="46"/>
       <x:c r="F128" s="46"/>
@@ -2968,11 +3240,13 @@
       <x:c r="M128" s="46"/>
       <x:c r="N128" s="46"/>
       <x:c r="O128" s="58"/>
+      <x:c r="P128" s="58"/>
+      <x:c r="Q128" s="61"/>
     </x:row>
     <x:row r="129" ht="15" hidden="0" customHeight="1">
       <x:c r="A129" s="52"/>
       <x:c r="B129" s="46"/>
-      <x:c r="C129" s="61"/>
+      <x:c r="C129" s="64"/>
       <x:c r="D129" s="55"/>
       <x:c r="E129" s="46"/>
       <x:c r="F129" s="46"/>
@@ -2985,11 +3259,13 @@
       <x:c r="M129" s="46"/>
       <x:c r="N129" s="46"/>
       <x:c r="O129" s="58"/>
+      <x:c r="P129" s="58"/>
+      <x:c r="Q129" s="61"/>
     </x:row>
     <x:row r="130" ht="15" hidden="0" customHeight="1">
       <x:c r="A130" s="52"/>
       <x:c r="B130" s="46"/>
-      <x:c r="C130" s="61"/>
+      <x:c r="C130" s="64"/>
       <x:c r="D130" s="55"/>
       <x:c r="E130" s="46"/>
       <x:c r="F130" s="46"/>
@@ -3002,11 +3278,13 @@
       <x:c r="M130" s="46"/>
       <x:c r="N130" s="46"/>
       <x:c r="O130" s="58"/>
+      <x:c r="P130" s="58"/>
+      <x:c r="Q130" s="61"/>
     </x:row>
     <x:row r="131" ht="15" hidden="0" customHeight="1">
       <x:c r="A131" s="52"/>
       <x:c r="B131" s="46"/>
-      <x:c r="C131" s="61"/>
+      <x:c r="C131" s="64"/>
       <x:c r="D131" s="55"/>
       <x:c r="E131" s="46"/>
       <x:c r="F131" s="46"/>
@@ -3019,11 +3297,13 @@
       <x:c r="M131" s="46"/>
       <x:c r="N131" s="46"/>
       <x:c r="O131" s="58"/>
+      <x:c r="P131" s="58"/>
+      <x:c r="Q131" s="61"/>
     </x:row>
     <x:row r="132" ht="15" hidden="0" customHeight="1">
       <x:c r="A132" s="52"/>
       <x:c r="B132" s="46"/>
-      <x:c r="C132" s="61"/>
+      <x:c r="C132" s="64"/>
       <x:c r="D132" s="55"/>
       <x:c r="E132" s="46"/>
       <x:c r="F132" s="46"/>
@@ -3036,11 +3316,13 @@
       <x:c r="M132" s="46"/>
       <x:c r="N132" s="46"/>
       <x:c r="O132" s="58"/>
+      <x:c r="P132" s="58"/>
+      <x:c r="Q132" s="61"/>
     </x:row>
     <x:row r="133" ht="15" hidden="0" customHeight="1">
       <x:c r="A133" s="52"/>
       <x:c r="B133" s="46"/>
-      <x:c r="C133" s="61"/>
+      <x:c r="C133" s="64"/>
       <x:c r="D133" s="55"/>
       <x:c r="E133" s="46"/>
       <x:c r="F133" s="46"/>
@@ -3053,11 +3335,13 @@
       <x:c r="M133" s="46"/>
       <x:c r="N133" s="46"/>
       <x:c r="O133" s="58"/>
+      <x:c r="P133" s="58"/>
+      <x:c r="Q133" s="61"/>
     </x:row>
     <x:row r="134" ht="15" hidden="0" customHeight="1">
       <x:c r="A134" s="52"/>
       <x:c r="B134" s="46"/>
-      <x:c r="C134" s="61"/>
+      <x:c r="C134" s="64"/>
       <x:c r="D134" s="55"/>
       <x:c r="E134" s="46"/>
       <x:c r="F134" s="46"/>
@@ -3070,11 +3354,13 @@
       <x:c r="M134" s="46"/>
       <x:c r="N134" s="46"/>
       <x:c r="O134" s="58"/>
+      <x:c r="P134" s="58"/>
+      <x:c r="Q134" s="61"/>
     </x:row>
     <x:row r="135" ht="15" hidden="0" customHeight="1">
       <x:c r="A135" s="52"/>
       <x:c r="B135" s="46"/>
-      <x:c r="C135" s="61"/>
+      <x:c r="C135" s="64"/>
       <x:c r="D135" s="55"/>
       <x:c r="E135" s="46"/>
       <x:c r="F135" s="46"/>
@@ -3087,11 +3373,13 @@
       <x:c r="M135" s="46"/>
       <x:c r="N135" s="46"/>
       <x:c r="O135" s="58"/>
+      <x:c r="P135" s="58"/>
+      <x:c r="Q135" s="61"/>
     </x:row>
     <x:row r="136" ht="15" hidden="0" customHeight="1">
       <x:c r="A136" s="52"/>
       <x:c r="B136" s="46"/>
-      <x:c r="C136" s="61"/>
+      <x:c r="C136" s="64"/>
       <x:c r="D136" s="55"/>
       <x:c r="E136" s="46"/>
       <x:c r="F136" s="46"/>
@@ -3104,11 +3392,13 @@
       <x:c r="M136" s="46"/>
       <x:c r="N136" s="46"/>
       <x:c r="O136" s="58"/>
+      <x:c r="P136" s="58"/>
+      <x:c r="Q136" s="61"/>
     </x:row>
     <x:row r="137" ht="15" hidden="0" customHeight="1">
       <x:c r="A137" s="52"/>
       <x:c r="B137" s="46"/>
-      <x:c r="C137" s="61"/>
+      <x:c r="C137" s="64"/>
       <x:c r="D137" s="55"/>
       <x:c r="E137" s="46"/>
       <x:c r="F137" s="46"/>
@@ -3121,11 +3411,13 @@
       <x:c r="M137" s="46"/>
       <x:c r="N137" s="46"/>
       <x:c r="O137" s="58"/>
+      <x:c r="P137" s="58"/>
+      <x:c r="Q137" s="61"/>
     </x:row>
     <x:row r="138" ht="15" hidden="0" customHeight="1">
       <x:c r="A138" s="52"/>
       <x:c r="B138" s="46"/>
-      <x:c r="C138" s="61"/>
+      <x:c r="C138" s="64"/>
       <x:c r="D138" s="55"/>
       <x:c r="E138" s="46"/>
       <x:c r="F138" s="46"/>
@@ -3138,11 +3430,13 @@
       <x:c r="M138" s="46"/>
       <x:c r="N138" s="46"/>
       <x:c r="O138" s="58"/>
+      <x:c r="P138" s="58"/>
+      <x:c r="Q138" s="61"/>
     </x:row>
     <x:row r="139" ht="15" hidden="0" customHeight="1">
       <x:c r="A139" s="52"/>
       <x:c r="B139" s="46"/>
-      <x:c r="C139" s="61"/>
+      <x:c r="C139" s="64"/>
       <x:c r="D139" s="55"/>
       <x:c r="E139" s="46"/>
       <x:c r="F139" s="46"/>
@@ -3155,11 +3449,13 @@
       <x:c r="M139" s="46"/>
       <x:c r="N139" s="46"/>
       <x:c r="O139" s="58"/>
+      <x:c r="P139" s="58"/>
+      <x:c r="Q139" s="61"/>
     </x:row>
     <x:row r="140" ht="15" hidden="0" customHeight="1">
       <x:c r="A140" s="52"/>
       <x:c r="B140" s="46"/>
-      <x:c r="C140" s="61"/>
+      <x:c r="C140" s="64"/>
       <x:c r="D140" s="55"/>
       <x:c r="E140" s="46"/>
       <x:c r="F140" s="46"/>
@@ -3172,11 +3468,13 @@
       <x:c r="M140" s="46"/>
       <x:c r="N140" s="46"/>
       <x:c r="O140" s="58"/>
+      <x:c r="P140" s="58"/>
+      <x:c r="Q140" s="61"/>
     </x:row>
     <x:row r="141" ht="15" hidden="0" customHeight="1">
       <x:c r="A141" s="52"/>
       <x:c r="B141" s="46"/>
-      <x:c r="C141" s="61"/>
+      <x:c r="C141" s="64"/>
       <x:c r="D141" s="55"/>
       <x:c r="E141" s="46"/>
       <x:c r="F141" s="46"/>
@@ -3189,11 +3487,13 @@
       <x:c r="M141" s="46"/>
       <x:c r="N141" s="46"/>
       <x:c r="O141" s="58"/>
+      <x:c r="P141" s="58"/>
+      <x:c r="Q141" s="61"/>
     </x:row>
     <x:row r="142" ht="15" hidden="0" customHeight="1">
       <x:c r="A142" s="52"/>
       <x:c r="B142" s="46"/>
-      <x:c r="C142" s="61"/>
+      <x:c r="C142" s="64"/>
       <x:c r="D142" s="55"/>
       <x:c r="E142" s="46"/>
       <x:c r="F142" s="46"/>
@@ -3206,11 +3506,13 @@
       <x:c r="M142" s="46"/>
       <x:c r="N142" s="46"/>
       <x:c r="O142" s="58"/>
+      <x:c r="P142" s="58"/>
+      <x:c r="Q142" s="61"/>
     </x:row>
     <x:row r="143" ht="15" hidden="0" customHeight="1">
       <x:c r="A143" s="52"/>
       <x:c r="B143" s="46"/>
-      <x:c r="C143" s="61"/>
+      <x:c r="C143" s="64"/>
       <x:c r="D143" s="55"/>
       <x:c r="E143" s="46"/>
       <x:c r="F143" s="46"/>
@@ -3223,11 +3525,13 @@
       <x:c r="M143" s="46"/>
       <x:c r="N143" s="46"/>
       <x:c r="O143" s="58"/>
+      <x:c r="P143" s="58"/>
+      <x:c r="Q143" s="61"/>
     </x:row>
     <x:row r="144" ht="15" hidden="0" customHeight="1">
       <x:c r="A144" s="52"/>
       <x:c r="B144" s="46"/>
-      <x:c r="C144" s="61"/>
+      <x:c r="C144" s="64"/>
       <x:c r="D144" s="55"/>
       <x:c r="E144" s="46"/>
       <x:c r="F144" s="46"/>
@@ -3240,11 +3544,13 @@
       <x:c r="M144" s="46"/>
       <x:c r="N144" s="46"/>
       <x:c r="O144" s="58"/>
+      <x:c r="P144" s="58"/>
+      <x:c r="Q144" s="61"/>
     </x:row>
     <x:row r="145" ht="15" hidden="0" customHeight="1">
       <x:c r="A145" s="52"/>
       <x:c r="B145" s="46"/>
-      <x:c r="C145" s="61"/>
+      <x:c r="C145" s="64"/>
       <x:c r="D145" s="55"/>
       <x:c r="E145" s="46"/>
       <x:c r="F145" s="46"/>
@@ -3257,11 +3563,13 @@
       <x:c r="M145" s="46"/>
       <x:c r="N145" s="46"/>
       <x:c r="O145" s="58"/>
+      <x:c r="P145" s="58"/>
+      <x:c r="Q145" s="61"/>
     </x:row>
     <x:row r="146" ht="15" hidden="0" customHeight="1">
       <x:c r="A146" s="52"/>
       <x:c r="B146" s="46"/>
-      <x:c r="C146" s="61"/>
+      <x:c r="C146" s="64"/>
       <x:c r="D146" s="55"/>
       <x:c r="E146" s="46"/>
       <x:c r="F146" s="46"/>
@@ -3274,11 +3582,13 @@
       <x:c r="M146" s="46"/>
       <x:c r="N146" s="46"/>
       <x:c r="O146" s="58"/>
+      <x:c r="P146" s="58"/>
+      <x:c r="Q146" s="61"/>
     </x:row>
     <x:row r="147" ht="15" hidden="0" customHeight="1">
       <x:c r="A147" s="52"/>
       <x:c r="B147" s="46"/>
-      <x:c r="C147" s="61"/>
+      <x:c r="C147" s="64"/>
       <x:c r="D147" s="55"/>
       <x:c r="E147" s="46"/>
       <x:c r="F147" s="46"/>
@@ -3291,11 +3601,13 @@
       <x:c r="M147" s="46"/>
       <x:c r="N147" s="46"/>
       <x:c r="O147" s="58"/>
+      <x:c r="P147" s="58"/>
+      <x:c r="Q147" s="61"/>
     </x:row>
     <x:row r="148" ht="15" hidden="0" customHeight="1">
       <x:c r="A148" s="52"/>
       <x:c r="B148" s="46"/>
-      <x:c r="C148" s="61"/>
+      <x:c r="C148" s="64"/>
       <x:c r="D148" s="55"/>
       <x:c r="E148" s="46"/>
       <x:c r="F148" s="46"/>
@@ -3308,11 +3620,13 @@
       <x:c r="M148" s="46"/>
       <x:c r="N148" s="46"/>
       <x:c r="O148" s="58"/>
+      <x:c r="P148" s="58"/>
+      <x:c r="Q148" s="61"/>
     </x:row>
     <x:row r="149" ht="15" hidden="0" customHeight="1">
       <x:c r="A149" s="52"/>
       <x:c r="B149" s="46"/>
-      <x:c r="C149" s="61"/>
+      <x:c r="C149" s="64"/>
       <x:c r="D149" s="55"/>
       <x:c r="E149" s="46"/>
       <x:c r="F149" s="46"/>
@@ -3325,11 +3639,13 @@
       <x:c r="M149" s="46"/>
       <x:c r="N149" s="46"/>
       <x:c r="O149" s="58"/>
+      <x:c r="P149" s="58"/>
+      <x:c r="Q149" s="61"/>
     </x:row>
     <x:row r="150" ht="15" hidden="0" customHeight="1">
       <x:c r="A150" s="52"/>
       <x:c r="B150" s="46"/>
-      <x:c r="C150" s="61"/>
+      <x:c r="C150" s="64"/>
       <x:c r="D150" s="55"/>
       <x:c r="E150" s="46"/>
       <x:c r="F150" s="46"/>
@@ -3342,11 +3658,13 @@
       <x:c r="M150" s="46"/>
       <x:c r="N150" s="46"/>
       <x:c r="O150" s="58"/>
+      <x:c r="P150" s="58"/>
+      <x:c r="Q150" s="61"/>
     </x:row>
     <x:row r="151" ht="15" hidden="0" customHeight="1">
       <x:c r="A151" s="52"/>
       <x:c r="B151" s="46"/>
-      <x:c r="C151" s="61"/>
+      <x:c r="C151" s="64"/>
       <x:c r="D151" s="55"/>
       <x:c r="E151" s="46"/>
       <x:c r="F151" s="46"/>
@@ -3359,11 +3677,13 @@
       <x:c r="M151" s="46"/>
       <x:c r="N151" s="46"/>
       <x:c r="O151" s="58"/>
+      <x:c r="P151" s="58"/>
+      <x:c r="Q151" s="61"/>
     </x:row>
     <x:row r="152" ht="15" hidden="0" customHeight="1">
       <x:c r="A152" s="52"/>
       <x:c r="B152" s="46"/>
-      <x:c r="C152" s="61"/>
+      <x:c r="C152" s="64"/>
       <x:c r="D152" s="55"/>
       <x:c r="E152" s="46"/>
       <x:c r="F152" s="46"/>
@@ -3376,11 +3696,13 @@
       <x:c r="M152" s="46"/>
       <x:c r="N152" s="46"/>
       <x:c r="O152" s="58"/>
+      <x:c r="P152" s="58"/>
+      <x:c r="Q152" s="61"/>
     </x:row>
     <x:row r="153" ht="15" hidden="0" customHeight="1">
       <x:c r="A153" s="52"/>
       <x:c r="B153" s="46"/>
-      <x:c r="C153" s="61"/>
+      <x:c r="C153" s="64"/>
       <x:c r="D153" s="55"/>
       <x:c r="E153" s="46"/>
       <x:c r="F153" s="46"/>
@@ -3393,11 +3715,13 @@
       <x:c r="M153" s="46"/>
       <x:c r="N153" s="46"/>
       <x:c r="O153" s="58"/>
+      <x:c r="P153" s="58"/>
+      <x:c r="Q153" s="61"/>
     </x:row>
     <x:row r="154" ht="15" hidden="0" customHeight="1">
       <x:c r="A154" s="52"/>
       <x:c r="B154" s="46"/>
-      <x:c r="C154" s="61"/>
+      <x:c r="C154" s="64"/>
       <x:c r="D154" s="55"/>
       <x:c r="E154" s="46"/>
       <x:c r="F154" s="46"/>
@@ -3410,11 +3734,13 @@
       <x:c r="M154" s="46"/>
       <x:c r="N154" s="46"/>
       <x:c r="O154" s="58"/>
+      <x:c r="P154" s="58"/>
+      <x:c r="Q154" s="61"/>
     </x:row>
     <x:row r="155" ht="15" hidden="0" customHeight="1">
       <x:c r="A155" s="52"/>
       <x:c r="B155" s="46"/>
-      <x:c r="C155" s="61"/>
+      <x:c r="C155" s="64"/>
       <x:c r="D155" s="55"/>
       <x:c r="E155" s="46"/>
       <x:c r="F155" s="46"/>
@@ -3427,11 +3753,13 @@
       <x:c r="M155" s="46"/>
       <x:c r="N155" s="46"/>
       <x:c r="O155" s="58"/>
+      <x:c r="P155" s="58"/>
+      <x:c r="Q155" s="61"/>
     </x:row>
     <x:row r="156" ht="15" hidden="0" customHeight="1">
       <x:c r="A156" s="52"/>
       <x:c r="B156" s="46"/>
-      <x:c r="C156" s="61"/>
+      <x:c r="C156" s="64"/>
       <x:c r="D156" s="55"/>
       <x:c r="E156" s="46"/>
       <x:c r="F156" s="46"/>
@@ -3444,11 +3772,13 @@
       <x:c r="M156" s="46"/>
       <x:c r="N156" s="46"/>
       <x:c r="O156" s="58"/>
+      <x:c r="P156" s="58"/>
+      <x:c r="Q156" s="61"/>
     </x:row>
     <x:row r="157" ht="15" hidden="0" customHeight="1">
       <x:c r="A157" s="52"/>
       <x:c r="B157" s="46"/>
-      <x:c r="C157" s="61"/>
+      <x:c r="C157" s="64"/>
       <x:c r="D157" s="55"/>
       <x:c r="E157" s="46"/>
       <x:c r="F157" s="46"/>
@@ -3461,11 +3791,13 @@
       <x:c r="M157" s="46"/>
       <x:c r="N157" s="46"/>
       <x:c r="O157" s="58"/>
+      <x:c r="P157" s="58"/>
+      <x:c r="Q157" s="61"/>
     </x:row>
     <x:row r="158" ht="15" hidden="0" customHeight="1">
       <x:c r="A158" s="52"/>
       <x:c r="B158" s="46"/>
-      <x:c r="C158" s="61"/>
+      <x:c r="C158" s="64"/>
       <x:c r="D158" s="55"/>
       <x:c r="E158" s="46"/>
       <x:c r="F158" s="46"/>
@@ -3478,11 +3810,13 @@
       <x:c r="M158" s="46"/>
       <x:c r="N158" s="46"/>
       <x:c r="O158" s="58"/>
+      <x:c r="P158" s="58"/>
+      <x:c r="Q158" s="61"/>
     </x:row>
     <x:row r="159" ht="15" hidden="0" customHeight="1">
       <x:c r="A159" s="52"/>
       <x:c r="B159" s="46"/>
-      <x:c r="C159" s="61"/>
+      <x:c r="C159" s="64"/>
       <x:c r="D159" s="55"/>
       <x:c r="E159" s="46"/>
       <x:c r="F159" s="46"/>
@@ -3495,11 +3829,13 @@
       <x:c r="M159" s="46"/>
       <x:c r="N159" s="46"/>
       <x:c r="O159" s="58"/>
+      <x:c r="P159" s="58"/>
+      <x:c r="Q159" s="61"/>
     </x:row>
     <x:row r="160" ht="15" hidden="0" customHeight="1">
       <x:c r="A160" s="52"/>
       <x:c r="B160" s="46"/>
-      <x:c r="C160" s="61"/>
+      <x:c r="C160" s="64"/>
       <x:c r="D160" s="55"/>
       <x:c r="E160" s="46"/>
       <x:c r="F160" s="46"/>
@@ -3512,11 +3848,13 @@
       <x:c r="M160" s="46"/>
       <x:c r="N160" s="46"/>
       <x:c r="O160" s="58"/>
+      <x:c r="P160" s="58"/>
+      <x:c r="Q160" s="61"/>
     </x:row>
     <x:row r="161" ht="15" hidden="0" customHeight="1">
       <x:c r="A161" s="52"/>
       <x:c r="B161" s="46"/>
-      <x:c r="C161" s="61"/>
+      <x:c r="C161" s="64"/>
       <x:c r="D161" s="55"/>
       <x:c r="E161" s="46"/>
       <x:c r="F161" s="46"/>
@@ -3529,11 +3867,13 @@
       <x:c r="M161" s="46"/>
       <x:c r="N161" s="46"/>
       <x:c r="O161" s="58"/>
+      <x:c r="P161" s="58"/>
+      <x:c r="Q161" s="61"/>
     </x:row>
     <x:row r="162" ht="15" hidden="0" customHeight="1">
       <x:c r="A162" s="52"/>
       <x:c r="B162" s="46"/>
-      <x:c r="C162" s="61"/>
+      <x:c r="C162" s="64"/>
       <x:c r="D162" s="55"/>
       <x:c r="E162" s="46"/>
       <x:c r="F162" s="46"/>
@@ -3546,11 +3886,13 @@
       <x:c r="M162" s="46"/>
       <x:c r="N162" s="46"/>
       <x:c r="O162" s="58"/>
+      <x:c r="P162" s="58"/>
+      <x:c r="Q162" s="61"/>
     </x:row>
     <x:row r="163" ht="15" hidden="0" customHeight="1">
       <x:c r="A163" s="52"/>
       <x:c r="B163" s="46"/>
-      <x:c r="C163" s="61"/>
+      <x:c r="C163" s="64"/>
       <x:c r="D163" s="55"/>
       <x:c r="E163" s="46"/>
       <x:c r="F163" s="46"/>
@@ -3563,11 +3905,13 @@
       <x:c r="M163" s="46"/>
       <x:c r="N163" s="46"/>
       <x:c r="O163" s="58"/>
+      <x:c r="P163" s="58"/>
+      <x:c r="Q163" s="61"/>
     </x:row>
     <x:row r="164" ht="15" hidden="0" customHeight="1">
       <x:c r="A164" s="52"/>
       <x:c r="B164" s="46"/>
-      <x:c r="C164" s="61"/>
+      <x:c r="C164" s="64"/>
       <x:c r="D164" s="55"/>
       <x:c r="E164" s="46"/>
       <x:c r="F164" s="46"/>
@@ -3580,11 +3924,13 @@
       <x:c r="M164" s="46"/>
       <x:c r="N164" s="46"/>
       <x:c r="O164" s="58"/>
+      <x:c r="P164" s="58"/>
+      <x:c r="Q164" s="61"/>
     </x:row>
     <x:row r="165" ht="15" hidden="0" customHeight="1">
       <x:c r="A165" s="52"/>
       <x:c r="B165" s="46"/>
-      <x:c r="C165" s="61"/>
+      <x:c r="C165" s="64"/>
       <x:c r="D165" s="55"/>
       <x:c r="E165" s="46"/>
       <x:c r="F165" s="46"/>
@@ -3597,11 +3943,13 @@
       <x:c r="M165" s="46"/>
       <x:c r="N165" s="46"/>
       <x:c r="O165" s="58"/>
+      <x:c r="P165" s="58"/>
+      <x:c r="Q165" s="61"/>
     </x:row>
     <x:row r="166" ht="15" hidden="0" customHeight="1">
       <x:c r="A166" s="52"/>
       <x:c r="B166" s="46"/>
-      <x:c r="C166" s="61"/>
+      <x:c r="C166" s="64"/>
       <x:c r="D166" s="55"/>
       <x:c r="E166" s="46"/>
       <x:c r="F166" s="46"/>
@@ -3614,11 +3962,13 @@
       <x:c r="M166" s="46"/>
       <x:c r="N166" s="46"/>
       <x:c r="O166" s="58"/>
+      <x:c r="P166" s="58"/>
+      <x:c r="Q166" s="61"/>
     </x:row>
     <x:row r="167" ht="15" hidden="0" customHeight="1">
       <x:c r="A167" s="52"/>
       <x:c r="B167" s="46"/>
-      <x:c r="C167" s="61"/>
+      <x:c r="C167" s="64"/>
       <x:c r="D167" s="55"/>
       <x:c r="E167" s="46"/>
       <x:c r="F167" s="46"/>
@@ -3631,11 +3981,13 @@
       <x:c r="M167" s="46"/>
       <x:c r="N167" s="46"/>
       <x:c r="O167" s="58"/>
+      <x:c r="P167" s="58"/>
+      <x:c r="Q167" s="61"/>
     </x:row>
     <x:row r="168" ht="15" hidden="0" customHeight="1">
       <x:c r="A168" s="52"/>
       <x:c r="B168" s="46"/>
-      <x:c r="C168" s="61"/>
+      <x:c r="C168" s="64"/>
       <x:c r="D168" s="55"/>
       <x:c r="E168" s="46"/>
       <x:c r="F168" s="46"/>
@@ -3648,11 +4000,13 @@
       <x:c r="M168" s="46"/>
       <x:c r="N168" s="46"/>
       <x:c r="O168" s="58"/>
+      <x:c r="P168" s="58"/>
+      <x:c r="Q168" s="61"/>
     </x:row>
     <x:row r="169" ht="15" hidden="0" customHeight="1">
       <x:c r="A169" s="52"/>
       <x:c r="B169" s="46"/>
-      <x:c r="C169" s="61"/>
+      <x:c r="C169" s="64"/>
       <x:c r="D169" s="55"/>
       <x:c r="E169" s="46"/>
       <x:c r="F169" s="46"/>
@@ -3665,11 +4019,13 @@
       <x:c r="M169" s="46"/>
       <x:c r="N169" s="46"/>
       <x:c r="O169" s="58"/>
+      <x:c r="P169" s="58"/>
+      <x:c r="Q169" s="61"/>
     </x:row>
     <x:row r="170" ht="15" hidden="0" customHeight="1">
       <x:c r="A170" s="52"/>
       <x:c r="B170" s="46"/>
-      <x:c r="C170" s="61"/>
+      <x:c r="C170" s="64"/>
       <x:c r="D170" s="55"/>
       <x:c r="E170" s="46"/>
       <x:c r="F170" s="46"/>
@@ -3682,11 +4038,13 @@
       <x:c r="M170" s="46"/>
       <x:c r="N170" s="46"/>
       <x:c r="O170" s="58"/>
+      <x:c r="P170" s="58"/>
+      <x:c r="Q170" s="61"/>
     </x:row>
     <x:row r="171" ht="15" hidden="0" customHeight="1">
       <x:c r="A171" s="52"/>
       <x:c r="B171" s="46"/>
-      <x:c r="C171" s="61"/>
+      <x:c r="C171" s="64"/>
       <x:c r="D171" s="55"/>
       <x:c r="E171" s="46"/>
       <x:c r="F171" s="46"/>
@@ -3699,11 +4057,13 @@
       <x:c r="M171" s="46"/>
       <x:c r="N171" s="46"/>
       <x:c r="O171" s="58"/>
+      <x:c r="P171" s="58"/>
+      <x:c r="Q171" s="61"/>
     </x:row>
     <x:row r="172" ht="15" hidden="0" customHeight="1">
       <x:c r="A172" s="52"/>
       <x:c r="B172" s="46"/>
-      <x:c r="C172" s="61"/>
+      <x:c r="C172" s="64"/>
       <x:c r="D172" s="55"/>
       <x:c r="E172" s="46"/>
       <x:c r="F172" s="46"/>
@@ -3716,11 +4076,13 @@
       <x:c r="M172" s="46"/>
       <x:c r="N172" s="46"/>
       <x:c r="O172" s="58"/>
+      <x:c r="P172" s="58"/>
+      <x:c r="Q172" s="61"/>
     </x:row>
     <x:row r="173" ht="15" hidden="0" customHeight="1">
       <x:c r="A173" s="52"/>
       <x:c r="B173" s="46"/>
-      <x:c r="C173" s="61"/>
+      <x:c r="C173" s="64"/>
       <x:c r="D173" s="55"/>
       <x:c r="E173" s="46"/>
       <x:c r="F173" s="46"/>
@@ -3733,11 +4095,13 @@
       <x:c r="M173" s="46"/>
       <x:c r="N173" s="46"/>
       <x:c r="O173" s="58"/>
+      <x:c r="P173" s="58"/>
+      <x:c r="Q173" s="61"/>
     </x:row>
     <x:row r="174" ht="15" hidden="0" customHeight="1">
       <x:c r="A174" s="52"/>
       <x:c r="B174" s="46"/>
-      <x:c r="C174" s="61"/>
+      <x:c r="C174" s="64"/>
       <x:c r="D174" s="55"/>
       <x:c r="E174" s="46"/>
       <x:c r="F174" s="46"/>
@@ -3750,11 +4114,13 @@
       <x:c r="M174" s="46"/>
       <x:c r="N174" s="46"/>
       <x:c r="O174" s="58"/>
+      <x:c r="P174" s="58"/>
+      <x:c r="Q174" s="61"/>
     </x:row>
     <x:row r="175" ht="15" hidden="0" customHeight="1">
       <x:c r="A175" s="52"/>
       <x:c r="B175" s="46"/>
-      <x:c r="C175" s="61"/>
+      <x:c r="C175" s="64"/>
       <x:c r="D175" s="55"/>
       <x:c r="E175" s="46"/>
       <x:c r="F175" s="46"/>
@@ -3767,11 +4133,13 @@
       <x:c r="M175" s="46"/>
       <x:c r="N175" s="46"/>
       <x:c r="O175" s="58"/>
+      <x:c r="P175" s="58"/>
+      <x:c r="Q175" s="61"/>
     </x:row>
     <x:row r="176" ht="15" hidden="0" customHeight="1">
       <x:c r="A176" s="52"/>
       <x:c r="B176" s="46"/>
-      <x:c r="C176" s="61"/>
+      <x:c r="C176" s="64"/>
       <x:c r="D176" s="55"/>
       <x:c r="E176" s="46"/>
       <x:c r="F176" s="46"/>
@@ -3784,11 +4152,13 @@
       <x:c r="M176" s="46"/>
       <x:c r="N176" s="46"/>
       <x:c r="O176" s="58"/>
+      <x:c r="P176" s="58"/>
+      <x:c r="Q176" s="61"/>
     </x:row>
     <x:row r="177" ht="15" hidden="0" customHeight="1">
       <x:c r="A177" s="52"/>
       <x:c r="B177" s="46"/>
-      <x:c r="C177" s="61"/>
+      <x:c r="C177" s="64"/>
       <x:c r="D177" s="55"/>
       <x:c r="E177" s="46"/>
       <x:c r="F177" s="46"/>
@@ -3801,11 +4171,13 @@
       <x:c r="M177" s="46"/>
       <x:c r="N177" s="46"/>
       <x:c r="O177" s="58"/>
+      <x:c r="P177" s="58"/>
+      <x:c r="Q177" s="61"/>
     </x:row>
     <x:row r="178" ht="15" hidden="0" customHeight="1">
       <x:c r="A178" s="52"/>
       <x:c r="B178" s="46"/>
-      <x:c r="C178" s="61"/>
+      <x:c r="C178" s="64"/>
       <x:c r="D178" s="55"/>
       <x:c r="E178" s="46"/>
       <x:c r="F178" s="46"/>
@@ -3818,11 +4190,13 @@
       <x:c r="M178" s="46"/>
       <x:c r="N178" s="46"/>
       <x:c r="O178" s="58"/>
+      <x:c r="P178" s="58"/>
+      <x:c r="Q178" s="61"/>
     </x:row>
     <x:row r="179" ht="15" hidden="0" customHeight="1">
       <x:c r="A179" s="52"/>
       <x:c r="B179" s="46"/>
-      <x:c r="C179" s="61"/>
+      <x:c r="C179" s="64"/>
       <x:c r="D179" s="55"/>
       <x:c r="E179" s="46"/>
       <x:c r="F179" s="46"/>
@@ -3835,11 +4209,13 @@
       <x:c r="M179" s="46"/>
       <x:c r="N179" s="46"/>
       <x:c r="O179" s="58"/>
+      <x:c r="P179" s="58"/>
+      <x:c r="Q179" s="61"/>
     </x:row>
     <x:row r="180" ht="15" hidden="0" customHeight="1">
       <x:c r="A180" s="52"/>
       <x:c r="B180" s="46"/>
-      <x:c r="C180" s="61"/>
+      <x:c r="C180" s="64"/>
       <x:c r="D180" s="55"/>
       <x:c r="E180" s="46"/>
       <x:c r="F180" s="46"/>
@@ -3852,11 +4228,13 @@
       <x:c r="M180" s="46"/>
       <x:c r="N180" s="46"/>
       <x:c r="O180" s="58"/>
+      <x:c r="P180" s="58"/>
+      <x:c r="Q180" s="61"/>
     </x:row>
     <x:row r="181" ht="15" hidden="0" customHeight="1">
       <x:c r="A181" s="52"/>
       <x:c r="B181" s="46"/>
-      <x:c r="C181" s="61"/>
+      <x:c r="C181" s="64"/>
       <x:c r="D181" s="55"/>
       <x:c r="E181" s="46"/>
       <x:c r="F181" s="46"/>
@@ -3869,11 +4247,13 @@
       <x:c r="M181" s="46"/>
       <x:c r="N181" s="46"/>
       <x:c r="O181" s="58"/>
+      <x:c r="P181" s="58"/>
+      <x:c r="Q181" s="61"/>
     </x:row>
     <x:row r="182" ht="15" hidden="0" customHeight="1">
       <x:c r="A182" s="52"/>
       <x:c r="B182" s="46"/>
-      <x:c r="C182" s="61"/>
+      <x:c r="C182" s="64"/>
       <x:c r="D182" s="55"/>
       <x:c r="E182" s="46"/>
       <x:c r="F182" s="46"/>
@@ -3886,11 +4266,13 @@
       <x:c r="M182" s="46"/>
       <x:c r="N182" s="46"/>
       <x:c r="O182" s="58"/>
+      <x:c r="P182" s="58"/>
+      <x:c r="Q182" s="61"/>
     </x:row>
     <x:row r="183" ht="15" hidden="0" customHeight="1">
       <x:c r="A183" s="52"/>
       <x:c r="B183" s="46"/>
-      <x:c r="C183" s="61"/>
+      <x:c r="C183" s="64"/>
       <x:c r="D183" s="55"/>
       <x:c r="E183" s="46"/>
       <x:c r="F183" s="46"/>
@@ -3903,11 +4285,13 @@
       <x:c r="M183" s="46"/>
       <x:c r="N183" s="46"/>
       <x:c r="O183" s="58"/>
+      <x:c r="P183" s="58"/>
+      <x:c r="Q183" s="61"/>
     </x:row>
     <x:row r="184" ht="15" hidden="0" customHeight="1">
       <x:c r="A184" s="52"/>
       <x:c r="B184" s="46"/>
-      <x:c r="C184" s="61"/>
+      <x:c r="C184" s="64"/>
       <x:c r="D184" s="55"/>
       <x:c r="E184" s="46"/>
       <x:c r="F184" s="46"/>
@@ -3920,11 +4304,13 @@
       <x:c r="M184" s="46"/>
       <x:c r="N184" s="46"/>
       <x:c r="O184" s="58"/>
+      <x:c r="P184" s="58"/>
+      <x:c r="Q184" s="61"/>
     </x:row>
     <x:row r="185" ht="15" hidden="0" customHeight="1">
       <x:c r="A185" s="52"/>
       <x:c r="B185" s="46"/>
-      <x:c r="C185" s="61"/>
+      <x:c r="C185" s="64"/>
       <x:c r="D185" s="55"/>
       <x:c r="E185" s="46"/>
       <x:c r="F185" s="46"/>
@@ -3937,11 +4323,13 @@
       <x:c r="M185" s="46"/>
       <x:c r="N185" s="46"/>
       <x:c r="O185" s="58"/>
+      <x:c r="P185" s="58"/>
+      <x:c r="Q185" s="61"/>
     </x:row>
     <x:row r="186" ht="15" hidden="0" customHeight="1">
       <x:c r="A186" s="52"/>
       <x:c r="B186" s="46"/>
-      <x:c r="C186" s="61"/>
+      <x:c r="C186" s="64"/>
       <x:c r="D186" s="55"/>
       <x:c r="E186" s="46"/>
       <x:c r="F186" s="46"/>
@@ -3954,11 +4342,13 @@
       <x:c r="M186" s="46"/>
       <x:c r="N186" s="46"/>
       <x:c r="O186" s="58"/>
+      <x:c r="P186" s="58"/>
+      <x:c r="Q186" s="61"/>
     </x:row>
     <x:row r="187" ht="15" hidden="0" customHeight="1">
       <x:c r="A187" s="52"/>
       <x:c r="B187" s="46"/>
-      <x:c r="C187" s="61"/>
+      <x:c r="C187" s="64"/>
       <x:c r="D187" s="55"/>
       <x:c r="E187" s="46"/>
       <x:c r="F187" s="46"/>
@@ -3971,11 +4361,13 @@
       <x:c r="M187" s="46"/>
       <x:c r="N187" s="46"/>
       <x:c r="O187" s="58"/>
+      <x:c r="P187" s="58"/>
+      <x:c r="Q187" s="61"/>
     </x:row>
     <x:row r="188" ht="15" hidden="0" customHeight="1">
       <x:c r="A188" s="52"/>
       <x:c r="B188" s="46"/>
-      <x:c r="C188" s="61"/>
+      <x:c r="C188" s="64"/>
       <x:c r="D188" s="55"/>
       <x:c r="E188" s="46"/>
       <x:c r="F188" s="46"/>
@@ -3988,11 +4380,13 @@
       <x:c r="M188" s="46"/>
       <x:c r="N188" s="46"/>
       <x:c r="O188" s="58"/>
+      <x:c r="P188" s="58"/>
+      <x:c r="Q188" s="61"/>
     </x:row>
     <x:row r="189" ht="15" hidden="0" customHeight="1">
       <x:c r="A189" s="52"/>
       <x:c r="B189" s="46"/>
-      <x:c r="C189" s="61"/>
+      <x:c r="C189" s="64"/>
       <x:c r="D189" s="55"/>
       <x:c r="E189" s="46"/>
       <x:c r="F189" s="46"/>
@@ -4005,11 +4399,13 @@
       <x:c r="M189" s="46"/>
       <x:c r="N189" s="46"/>
       <x:c r="O189" s="58"/>
+      <x:c r="P189" s="58"/>
+      <x:c r="Q189" s="61"/>
     </x:row>
     <x:row r="190" ht="15" hidden="0" customHeight="1">
       <x:c r="A190" s="52"/>
       <x:c r="B190" s="46"/>
-      <x:c r="C190" s="61"/>
+      <x:c r="C190" s="64"/>
       <x:c r="D190" s="55"/>
       <x:c r="E190" s="46"/>
       <x:c r="F190" s="46"/>
@@ -4022,11 +4418,13 @@
       <x:c r="M190" s="46"/>
       <x:c r="N190" s="46"/>
       <x:c r="O190" s="58"/>
+      <x:c r="P190" s="58"/>
+      <x:c r="Q190" s="61"/>
     </x:row>
     <x:row r="191" ht="15" hidden="0" customHeight="1">
       <x:c r="A191" s="52"/>
       <x:c r="B191" s="46"/>
-      <x:c r="C191" s="61"/>
+      <x:c r="C191" s="64"/>
       <x:c r="D191" s="55"/>
       <x:c r="E191" s="46"/>
       <x:c r="F191" s="46"/>
@@ -4039,11 +4437,13 @@
       <x:c r="M191" s="46"/>
       <x:c r="N191" s="46"/>
       <x:c r="O191" s="58"/>
+      <x:c r="P191" s="58"/>
+      <x:c r="Q191" s="61"/>
     </x:row>
     <x:row r="192" ht="15" hidden="0" customHeight="1">
       <x:c r="A192" s="52"/>
       <x:c r="B192" s="46"/>
-      <x:c r="C192" s="61"/>
+      <x:c r="C192" s="64"/>
       <x:c r="D192" s="55"/>
       <x:c r="E192" s="46"/>
       <x:c r="F192" s="46"/>
@@ -4056,11 +4456,13 @@
       <x:c r="M192" s="46"/>
       <x:c r="N192" s="46"/>
       <x:c r="O192" s="58"/>
+      <x:c r="P192" s="58"/>
+      <x:c r="Q192" s="61"/>
     </x:row>
     <x:row r="193" ht="15" hidden="0" customHeight="1">
       <x:c r="A193" s="52"/>
       <x:c r="B193" s="46"/>
-      <x:c r="C193" s="61"/>
+      <x:c r="C193" s="64"/>
       <x:c r="D193" s="55"/>
       <x:c r="E193" s="46"/>
       <x:c r="F193" s="46"/>
@@ -4073,11 +4475,13 @@
       <x:c r="M193" s="46"/>
       <x:c r="N193" s="46"/>
       <x:c r="O193" s="58"/>
+      <x:c r="P193" s="58"/>
+      <x:c r="Q193" s="61"/>
     </x:row>
     <x:row r="194" ht="15" hidden="0" customHeight="1">
       <x:c r="A194" s="52"/>
       <x:c r="B194" s="46"/>
-      <x:c r="C194" s="61"/>
+      <x:c r="C194" s="64"/>
       <x:c r="D194" s="55"/>
       <x:c r="E194" s="46"/>
       <x:c r="F194" s="46"/>
@@ -4090,11 +4494,13 @@
       <x:c r="M194" s="46"/>
       <x:c r="N194" s="46"/>
       <x:c r="O194" s="58"/>
+      <x:c r="P194" s="58"/>
+      <x:c r="Q194" s="61"/>
     </x:row>
     <x:row r="195" ht="15" hidden="0" customHeight="1">
       <x:c r="A195" s="52"/>
       <x:c r="B195" s="46"/>
-      <x:c r="C195" s="61"/>
+      <x:c r="C195" s="64"/>
       <x:c r="D195" s="55"/>
       <x:c r="E195" s="46"/>
       <x:c r="F195" s="46"/>
@@ -4107,11 +4513,13 @@
       <x:c r="M195" s="46"/>
       <x:c r="N195" s="46"/>
       <x:c r="O195" s="58"/>
+      <x:c r="P195" s="58"/>
+      <x:c r="Q195" s="61"/>
     </x:row>
     <x:row r="196" ht="15" hidden="0" customHeight="1">
       <x:c r="A196" s="52"/>
       <x:c r="B196" s="46"/>
-      <x:c r="C196" s="61"/>
+      <x:c r="C196" s="64"/>
       <x:c r="D196" s="55"/>
       <x:c r="E196" s="46"/>
       <x:c r="F196" s="46"/>
@@ -4124,11 +4532,13 @@
       <x:c r="M196" s="46"/>
       <x:c r="N196" s="46"/>
       <x:c r="O196" s="58"/>
+      <x:c r="P196" s="58"/>
+      <x:c r="Q196" s="61"/>
     </x:row>
     <x:row r="197" ht="15" hidden="0" customHeight="1">
       <x:c r="A197" s="52"/>
       <x:c r="B197" s="46"/>
-      <x:c r="C197" s="61"/>
+      <x:c r="C197" s="64"/>
       <x:c r="D197" s="55"/>
       <x:c r="E197" s="46"/>
       <x:c r="F197" s="46"/>
@@ -4141,11 +4551,13 @@
       <x:c r="M197" s="46"/>
       <x:c r="N197" s="46"/>
       <x:c r="O197" s="58"/>
+      <x:c r="P197" s="58"/>
+      <x:c r="Q197" s="61"/>
     </x:row>
     <x:row r="198" ht="15" hidden="0" customHeight="1">
       <x:c r="A198" s="52"/>
       <x:c r="B198" s="46"/>
-      <x:c r="C198" s="61"/>
+      <x:c r="C198" s="64"/>
       <x:c r="D198" s="55"/>
       <x:c r="E198" s="46"/>
       <x:c r="F198" s="46"/>
@@ -4158,11 +4570,13 @@
       <x:c r="M198" s="46"/>
       <x:c r="N198" s="46"/>
       <x:c r="O198" s="58"/>
+      <x:c r="P198" s="58"/>
+      <x:c r="Q198" s="61"/>
     </x:row>
     <x:row r="199" ht="15" hidden="0" customHeight="1">
       <x:c r="A199" s="52"/>
       <x:c r="B199" s="46"/>
-      <x:c r="C199" s="61"/>
+      <x:c r="C199" s="64"/>
       <x:c r="D199" s="55"/>
       <x:c r="E199" s="46"/>
       <x:c r="F199" s="46"/>
@@ -4175,11 +4589,13 @@
       <x:c r="M199" s="46"/>
       <x:c r="N199" s="46"/>
       <x:c r="O199" s="58"/>
+      <x:c r="P199" s="58"/>
+      <x:c r="Q199" s="61"/>
     </x:row>
     <x:row r="200" ht="15" hidden="0" customHeight="1">
       <x:c r="A200" s="52"/>
       <x:c r="B200" s="46"/>
-      <x:c r="C200" s="61"/>
+      <x:c r="C200" s="64"/>
       <x:c r="D200" s="55"/>
       <x:c r="E200" s="46"/>
       <x:c r="F200" s="46"/>
@@ -4192,11 +4608,13 @@
       <x:c r="M200" s="46"/>
       <x:c r="N200" s="46"/>
       <x:c r="O200" s="58"/>
+      <x:c r="P200" s="58"/>
+      <x:c r="Q200" s="61"/>
     </x:row>
     <x:row r="201" ht="15" hidden="0" customHeight="1">
       <x:c r="A201" s="52"/>
       <x:c r="B201" s="46"/>
-      <x:c r="C201" s="61"/>
+      <x:c r="C201" s="64"/>
       <x:c r="D201" s="55"/>
       <x:c r="E201" s="46"/>
       <x:c r="F201" s="46"/>
@@ -4209,11 +4627,13 @@
       <x:c r="M201" s="46"/>
       <x:c r="N201" s="46"/>
       <x:c r="O201" s="58"/>
+      <x:c r="P201" s="58"/>
+      <x:c r="Q201" s="61"/>
     </x:row>
     <x:row r="202" ht="15" hidden="0" customHeight="1">
       <x:c r="A202" s="52"/>
       <x:c r="B202" s="46"/>
-      <x:c r="C202" s="61"/>
+      <x:c r="C202" s="64"/>
       <x:c r="D202" s="55"/>
       <x:c r="E202" s="46"/>
       <x:c r="F202" s="46"/>
@@ -4226,11 +4646,13 @@
       <x:c r="M202" s="46"/>
       <x:c r="N202" s="46"/>
       <x:c r="O202" s="58"/>
+      <x:c r="P202" s="58"/>
+      <x:c r="Q202" s="61"/>
     </x:row>
     <x:row r="203" ht="15" hidden="0" customHeight="1">
       <x:c r="A203" s="52"/>
       <x:c r="B203" s="46"/>
-      <x:c r="C203" s="61"/>
+      <x:c r="C203" s="64"/>
       <x:c r="D203" s="55"/>
       <x:c r="E203" s="46"/>
       <x:c r="F203" s="46"/>
@@ -4243,11 +4665,13 @@
       <x:c r="M203" s="46"/>
       <x:c r="N203" s="46"/>
       <x:c r="O203" s="58"/>
+      <x:c r="P203" s="58"/>
+      <x:c r="Q203" s="61"/>
     </x:row>
     <x:row r="204" ht="15" hidden="0" customHeight="1">
       <x:c r="A204" s="53"/>
       <x:c r="B204" s="49"/>
-      <x:c r="C204" s="62"/>
+      <x:c r="C204" s="65"/>
       <x:c r="D204" s="56"/>
       <x:c r="E204" s="49"/>
       <x:c r="F204" s="49"/>
@@ -4260,11 +4684,13 @@
       <x:c r="M204" s="49"/>
       <x:c r="N204" s="49"/>
       <x:c r="O204" s="59"/>
+      <x:c r="P204" s="59"/>
+      <x:c r="Q204" s="62"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:O1"/>
-    <x:mergeCell ref="A2:O2"/>
+    <x:mergeCell ref="A1:Q1"/>
+    <x:mergeCell ref="A2:Q2"/>
   </x:mergeCells>
   <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="A5:A204">
@@ -4305,159 +4731,199 @@
       <x:c r="F1" s="4"/>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
-      <x:c r="A3" s="65" t="str">
+      <x:c r="A3" s="68" t="str">
         <x:v>Campo</x:v>
       </x:c>
-      <x:c r="B3" s="65" t="str">
+      <x:c r="B3" s="68" t="str">
         <x:v>Obrigatório</x:v>
       </x:c>
-      <x:c r="C3" s="65" t="str">
+      <x:c r="C3" s="68" t="str">
         <x:v>Múltipla escolha</x:v>
       </x:c>
-      <x:c r="D3" s="65" t="str">
+      <x:c r="D3" s="68" t="str">
         <x:v>Verdadeiro ou falso</x:v>
       </x:c>
-      <x:c r="E3" s="65" t="str">
+      <x:c r="E3" s="68" t="str">
         <x:v>Dissertativa</x:v>
       </x:c>
-      <x:c r="F3" s="65" t="str">
+      <x:c r="F3" s="68" t="str">
         <x:v>Regra</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
-      <x:c r="A4" s="93" t="str">
+      <x:c r="A4" s="96" t="str">
         <x:v>Tipo</x:v>
       </x:c>
-      <x:c r="B4" s="85" t="str">
+      <x:c r="B4" s="88" t="str">
         <x:v>Sim</x:v>
       </x:c>
-      <x:c r="C4" s="85" t="str">
+      <x:c r="C4" s="88" t="str">
         <x:v>Múltipla escolha</x:v>
       </x:c>
-      <x:c r="D4" s="85" t="str">
+      <x:c r="D4" s="88" t="str">
         <x:v>Verdadeiro ou falso</x:v>
       </x:c>
-      <x:c r="E4" s="85" t="str">
+      <x:c r="E4" s="88" t="str">
         <x:v>Dissertativa</x:v>
       </x:c>
-      <x:c r="F4" s="86" t="str">
+      <x:c r="F4" s="89" t="str">
         <x:v>Selecione uma das três opções.</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
-      <x:c r="A5" s="94" t="str">
+      <x:c r="A5" s="97" t="str">
         <x:v>Enunciado</x:v>
       </x:c>
-      <x:c r="B5" s="88" t="str">
+      <x:c r="B5" s="91" t="str">
         <x:v>Sim</x:v>
       </x:c>
-      <x:c r="C5" s="88" t="str">
+      <x:c r="C5" s="91" t="str">
         <x:v>Texto da pergunta</x:v>
       </x:c>
-      <x:c r="D5" s="88" t="str">
+      <x:c r="D5" s="91" t="str">
         <x:v>Texto da afirmação</x:v>
       </x:c>
-      <x:c r="E5" s="88" t="str">
+      <x:c r="E5" s="91" t="str">
         <x:v>Texto da pergunta</x:v>
       </x:c>
-      <x:c r="F5" s="89" t="str">
+      <x:c r="F5" s="92" t="str">
         <x:v>Até 3.000 caracteres.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="94" t="str">
+      <x:c r="A6" s="97" t="str">
         <x:v>Pontos</x:v>
       </x:c>
-      <x:c r="B6" s="88" t="str">
+      <x:c r="B6" s="91" t="str">
         <x:v>Não</x:v>
       </x:c>
-      <x:c r="C6" s="88" t="str">
+      <x:c r="C6" s="91" t="str">
         <x:v>Número de 0 a 1000</x:v>
       </x:c>
-      <x:c r="D6" s="88" t="str">
+      <x:c r="D6" s="91" t="str">
         <x:v>Número de 0 a 1000</x:v>
       </x:c>
-      <x:c r="E6" s="88" t="str">
+      <x:c r="E6" s="91" t="str">
         <x:v>Número de 0 a 1000</x:v>
       </x:c>
-      <x:c r="F6" s="89" t="str">
+      <x:c r="F6" s="92" t="str">
         <x:v>Se vazio, o sistema usa 10 pontos.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
-      <x:c r="A7" s="94" t="str">
+      <x:c r="A7" s="97" t="str">
         <x:v>Obrigatória</x:v>
       </x:c>
-      <x:c r="B7" s="88" t="str">
+      <x:c r="B7" s="91" t="str">
         <x:v>Não</x:v>
       </x:c>
-      <x:c r="C7" s="88" t="str">
+      <x:c r="C7" s="91" t="str">
         <x:v>Sim ou Não</x:v>
       </x:c>
-      <x:c r="D7" s="88" t="str">
+      <x:c r="D7" s="91" t="str">
         <x:v>Sim ou Não</x:v>
       </x:c>
-      <x:c r="E7" s="88" t="str">
+      <x:c r="E7" s="91" t="str">
         <x:v>Sim ou Não</x:v>
       </x:c>
-      <x:c r="F7" s="89" t="str">
+      <x:c r="F7" s="92" t="str">
         <x:v>Se vazio, o sistema considera Sim.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
-      <x:c r="A8" s="94" t="str">
+      <x:c r="A8" s="97" t="str">
         <x:v>Alternativas</x:v>
       </x:c>
-      <x:c r="B8" s="88" t="str">
+      <x:c r="B8" s="91" t="str">
         <x:v>Sim</x:v>
       </x:c>
-      <x:c r="C8" s="88" t="str">
+      <x:c r="C8" s="91" t="str">
         <x:v>Preencha ao menos A e B</x:v>
       </x:c>
-      <x:c r="D8" s="88" t="str">
+      <x:c r="D8" s="91" t="str">
         <x:v>Não preencher</x:v>
       </x:c>
-      <x:c r="E8" s="88" t="str">
+      <x:c r="E8" s="91" t="str">
         <x:v>Não preencher</x:v>
       </x:c>
-      <x:c r="F8" s="89" t="str">
+      <x:c r="F8" s="92" t="str">
         <x:v>São aceitas até dez alternativas.</x:v>
       </x:c>
     </x:row>
-    <x:row r="9" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A9" s="95" t="str">
+    <x:row r="9" ht="39.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A9" s="97" t="str">
+        <x:v>Imagem</x:v>
+      </x:c>
+      <x:c r="B9" s="91" t="str">
+        <x:v>Não</x:v>
+      </x:c>
+      <x:c r="C9" s="91" t="str">
+        <x:v>Link ou data:image</x:v>
+      </x:c>
+      <x:c r="D9" s="91" t="str">
+        <x:v>Link ou data:image</x:v>
+      </x:c>
+      <x:c r="E9" s="91" t="str">
+        <x:v>Link ou data:image</x:v>
+      </x:c>
+      <x:c r="F9" s="92" t="str">
+        <x:v>Use URL https:// ou data:image/png|jpeg|webp;base64. Também é possível anexar manualmente no editor.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
+      <x:c r="A10" s="97" t="str">
+        <x:v>Texto alternativo</x:v>
+      </x:c>
+      <x:c r="B10" s="91" t="str">
+        <x:v>Não</x:v>
+      </x:c>
+      <x:c r="C10" s="91" t="str">
+        <x:v>Descrição da imagem</x:v>
+      </x:c>
+      <x:c r="D10" s="91" t="str">
+        <x:v>Descrição da imagem</x:v>
+      </x:c>
+      <x:c r="E10" s="91" t="str">
+        <x:v>Descrição da imagem</x:v>
+      </x:c>
+      <x:c r="F10" s="92" t="str">
+        <x:v>Ajuda acessibilidade e revisão da questão.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="26.399999618530273" hidden="0" customHeight="1">
+      <x:c r="A11" s="98" t="str">
         <x:v>Resposta correta</x:v>
       </x:c>
-      <x:c r="B9" s="91" t="str">
+      <x:c r="B11" s="94" t="str">
         <x:v>Sim*</x:v>
       </x:c>
-      <x:c r="C9" s="91" t="str">
+      <x:c r="C11" s="94" t="str">
         <x:v>Texto exato ou letra da alternativa</x:v>
       </x:c>
-      <x:c r="D9" s="91" t="str">
+      <x:c r="D11" s="94" t="str">
         <x:v>Verdadeiro ou Falso</x:v>
       </x:c>
-      <x:c r="E9" s="91" t="str">
+      <x:c r="E11" s="94" t="str">
         <x:v>Opcional</x:v>
       </x:c>
-      <x:c r="F9" s="92" t="str">
+      <x:c r="F11" s="95" t="str">
         <x:v>*Obrigatória nas questões objetivas.</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="42" customHeight="1">
-      <x:c r="A11" s="99" t="str">
+    <x:row r="13" ht="42" customHeight="1">
+      <x:c r="A13" s="102" t="str">
         <x:v>IMPORTANTE: não renomeie a aba Questões nem altere os títulos das colunas. Salve o arquivo no formato .xlsx antes de importar.</x:v>
       </x:c>
-      <x:c r="B11" s="99"/>
-      <x:c r="C11" s="99"/>
-      <x:c r="D11" s="99"/>
-      <x:c r="E11" s="99"/>
-      <x:c r="F11" s="99"/>
+      <x:c r="B13" s="102"/>
+      <x:c r="C13" s="102"/>
+      <x:c r="D13" s="102"/>
+      <x:c r="E13" s="102"/>
+      <x:c r="F13" s="102"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:F1"/>
-    <x:mergeCell ref="A11:F11"/>
+    <x:mergeCell ref="A13:F13"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -4481,7 +4947,9 @@
     <x:col min="12" max="12" width="24" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="24" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="24" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="26" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="42" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="32" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="26" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
@@ -4502,142 +4970,160 @@
       <x:c r="M1" s="4"/>
       <x:c r="N1" s="4"/>
       <x:c r="O1" s="4"/>
+      <x:c r="P1" s="4"/>
+      <x:c r="Q1" s="4"/>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
-      <x:c r="A3" s="65" t="str">
+      <x:c r="A3" s="68" t="str">
         <x:v>Tipo</x:v>
       </x:c>
-      <x:c r="B3" s="65" t="str">
+      <x:c r="B3" s="68" t="str">
         <x:v>Enunciado</x:v>
       </x:c>
-      <x:c r="C3" s="65" t="str">
+      <x:c r="C3" s="68" t="str">
         <x:v>Pontos</x:v>
       </x:c>
-      <x:c r="D3" s="65" t="str">
+      <x:c r="D3" s="68" t="str">
         <x:v>Obrigatória</x:v>
       </x:c>
-      <x:c r="E3" s="65" t="str">
+      <x:c r="E3" s="68" t="str">
         <x:v>Alternativa A</x:v>
       </x:c>
-      <x:c r="F3" s="65" t="str">
+      <x:c r="F3" s="68" t="str">
         <x:v>Alternativa B</x:v>
       </x:c>
-      <x:c r="G3" s="65" t="str">
+      <x:c r="G3" s="68" t="str">
         <x:v>Alternativa C</x:v>
       </x:c>
-      <x:c r="H3" s="65" t="str">
+      <x:c r="H3" s="68" t="str">
         <x:v>Alternativa D</x:v>
       </x:c>
-      <x:c r="I3" s="65" t="str">
+      <x:c r="I3" s="68" t="str">
         <x:v>Alternativa E</x:v>
       </x:c>
-      <x:c r="J3" s="65" t="str">
+      <x:c r="J3" s="68" t="str">
         <x:v>Alternativa F</x:v>
       </x:c>
-      <x:c r="K3" s="65" t="str">
+      <x:c r="K3" s="68" t="str">
         <x:v>Alternativa G</x:v>
       </x:c>
-      <x:c r="L3" s="65" t="str">
+      <x:c r="L3" s="68" t="str">
         <x:v>Alternativa H</x:v>
       </x:c>
-      <x:c r="M3" s="65" t="str">
+      <x:c r="M3" s="68" t="str">
         <x:v>Alternativa I</x:v>
       </x:c>
-      <x:c r="N3" s="65" t="str">
+      <x:c r="N3" s="68" t="str">
         <x:v>Alternativa J</x:v>
       </x:c>
-      <x:c r="O3" s="65" t="str">
+      <x:c r="O3" s="68" t="str">
+        <x:v>Imagem</x:v>
+      </x:c>
+      <x:c r="P3" s="68" t="str">
+        <x:v>Texto alternativo</x:v>
+      </x:c>
+      <x:c r="Q3" s="68" t="str">
         <x:v>Resposta correta</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
-      <x:c r="A4" s="84" t="str">
+      <x:c r="A4" s="87" t="str">
         <x:v>Múltipla escolha</x:v>
       </x:c>
-      <x:c r="B4" s="85" t="str">
+      <x:c r="B4" s="88" t="str">
         <x:v>Qual alternativa representa uma comunicação clara?</x:v>
       </x:c>
-      <x:c r="C4" s="85" t="n">
+      <x:c r="C4" s="88" t="n">
         <x:v>20</x:v>
       </x:c>
-      <x:c r="D4" s="85" t="str">
+      <x:c r="D4" s="88" t="str">
         <x:v>Sim</x:v>
       </x:c>
-      <x:c r="E4" s="85" t="str">
+      <x:c r="E4" s="88" t="str">
         <x:v>Mensagem objetiva</x:v>
       </x:c>
-      <x:c r="F4" s="85" t="str">
+      <x:c r="F4" s="88" t="str">
         <x:v>Uso excessivo de termos técnicos</x:v>
       </x:c>
-      <x:c r="G4" s="85" t="str">
+      <x:c r="G4" s="88" t="str">
         <x:v>Ausência de retorno</x:v>
       </x:c>
-      <x:c r="H4" s="85" t="str"/>
-      <x:c r="I4" s="85" t="str"/>
-      <x:c r="J4" s="85" t="str"/>
-      <x:c r="K4" s="85" t="str"/>
-      <x:c r="L4" s="85" t="str"/>
-      <x:c r="M4" s="85" t="str"/>
-      <x:c r="N4" s="85" t="str"/>
-      <x:c r="O4" s="86" t="str">
+      <x:c r="H4" s="88" t="str"/>
+      <x:c r="I4" s="88" t="str"/>
+      <x:c r="J4" s="88" t="str"/>
+      <x:c r="K4" s="88" t="str"/>
+      <x:c r="L4" s="88" t="str"/>
+      <x:c r="M4" s="88" t="str"/>
+      <x:c r="N4" s="88" t="str"/>
+      <x:c r="O4" s="88" t="str">
+        <x:v>https://exemplo.com/grafico.png</x:v>
+      </x:c>
+      <x:c r="P4" s="88" t="str">
+        <x:v>Gráfico de apoio da questão</x:v>
+      </x:c>
+      <x:c r="Q4" s="89" t="str">
         <x:v>A</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
-      <x:c r="A5" s="87" t="str">
+      <x:c r="A5" s="90" t="str">
         <x:v>Verdadeiro ou falso</x:v>
       </x:c>
-      <x:c r="B5" s="88" t="str">
+      <x:c r="B5" s="91" t="str">
         <x:v>O feedback deve ser específico e respeitoso.</x:v>
       </x:c>
-      <x:c r="C5" s="88" t="n">
+      <x:c r="C5" s="91" t="n">
         <x:v>10</x:v>
       </x:c>
-      <x:c r="D5" s="88" t="str">
+      <x:c r="D5" s="91" t="str">
         <x:v>Sim</x:v>
       </x:c>
-      <x:c r="E5" s="88" t="str"/>
-      <x:c r="F5" s="88" t="str"/>
-      <x:c r="G5" s="88" t="str"/>
-      <x:c r="H5" s="88" t="str"/>
-      <x:c r="I5" s="88" t="str"/>
-      <x:c r="J5" s="88" t="str"/>
-      <x:c r="K5" s="88" t="str"/>
-      <x:c r="L5" s="88" t="str"/>
-      <x:c r="M5" s="88" t="str"/>
-      <x:c r="N5" s="88" t="str"/>
-      <x:c r="O5" s="89" t="str">
+      <x:c r="E5" s="91" t="str"/>
+      <x:c r="F5" s="91" t="str"/>
+      <x:c r="G5" s="91" t="str"/>
+      <x:c r="H5" s="91" t="str"/>
+      <x:c r="I5" s="91" t="str"/>
+      <x:c r="J5" s="91" t="str"/>
+      <x:c r="K5" s="91" t="str"/>
+      <x:c r="L5" s="91" t="str"/>
+      <x:c r="M5" s="91" t="str"/>
+      <x:c r="N5" s="91" t="str"/>
+      <x:c r="O5" s="91" t="str"/>
+      <x:c r="P5" s="91" t="str"/>
+      <x:c r="Q5" s="92" t="str">
         <x:v>Verdadeiro</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
-      <x:c r="A6" s="90" t="str">
+      <x:c r="A6" s="93" t="str">
         <x:v>Dissertativa</x:v>
       </x:c>
-      <x:c r="B6" s="91" t="str">
+      <x:c r="B6" s="94" t="str">
         <x:v>Descreva como você resolveria um conflito de equipe.</x:v>
       </x:c>
-      <x:c r="C6" s="91" t="n">
+      <x:c r="C6" s="94" t="n">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="D6" s="91" t="str">
+      <x:c r="D6" s="94" t="str">
         <x:v>Não</x:v>
       </x:c>
-      <x:c r="E6" s="91" t="str"/>
-      <x:c r="F6" s="91" t="str"/>
-      <x:c r="G6" s="91" t="str"/>
-      <x:c r="H6" s="91" t="str"/>
-      <x:c r="I6" s="91" t="str"/>
-      <x:c r="J6" s="91" t="str"/>
-      <x:c r="K6" s="91" t="str"/>
-      <x:c r="L6" s="91" t="str"/>
-      <x:c r="M6" s="91" t="str"/>
-      <x:c r="N6" s="91" t="str"/>
-      <x:c r="O6" s="92" t="str"/>
+      <x:c r="E6" s="94" t="str"/>
+      <x:c r="F6" s="94" t="str"/>
+      <x:c r="G6" s="94" t="str"/>
+      <x:c r="H6" s="94" t="str"/>
+      <x:c r="I6" s="94" t="str"/>
+      <x:c r="J6" s="94" t="str"/>
+      <x:c r="K6" s="94" t="str"/>
+      <x:c r="L6" s="94" t="str"/>
+      <x:c r="M6" s="94" t="str"/>
+      <x:c r="N6" s="94" t="str"/>
+      <x:c r="O6" s="94" t="str"/>
+      <x:c r="P6" s="94" t="str"/>
+      <x:c r="Q6" s="95" t="str"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:O1"/>
+    <x:mergeCell ref="A1:Q1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>